<commit_message>
feat: Enhance seed generation and image handling
- Added extractUrl function to handle URL extraction from various formats in Excel.
- Updated main function to read file path from command line argument.
- Improved image URL handling in product data by using extractUrl.
- Refactored image handling in AdminCataloguePanel to validate image URLs before rendering.
- Enhanced ProductFormModal to check for valid image URLs and provide appropriate placeholders.
- Added a new Excel file for export with updated data.
</commit_message>
<xml_diff>
--- a/chinni-treasure/exports/chinni-treasure-export-2026-07-18T18-45-09.xlsx
+++ b/chinni-treasure/exports/chinni-treasure-export-2026-07-18T18-45-09.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8B2DA7A-8C39-4F9C-89F9-78F17DAD1CCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{817BC37A-6F29-40F1-82BA-DC9129D204D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="541">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="542">
   <si>
     <t>ID</t>
   </si>
@@ -817,9 +817,6 @@
     <t>714879c0-acc2-4b7b-8a33-7c918ae9acf7</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/67pHD4f-IMG_20260705_174006.jpg</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
@@ -835,9 +832,6 @@
     <t>07d1cf51-7ecb-49cc-8b48-d69f4553a13f</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/yykLghU-IMG_20260705_174152.jpg</t>
-  </si>
-  <si>
     <t>943f5231-1014-4af5-ace3-632377a770e4</t>
   </si>
   <si>
@@ -847,9 +841,6 @@
     <t>bd99d7b7-1b7c-4933-b1e9-e7b0b5d41ae8</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/dcsEDNF-IMG_20260705_173922.jpg</t>
-  </si>
-  <si>
     <t>d9d6e26e-4dd7-4b82-b04f-c1fbe38f98a0</t>
   </si>
   <si>
@@ -1982,13 +1973,28 @@
   </si>
   <si>
     <t>Status changed to shipped</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/67pHD4f-IMG_20260705_174006.jpg</t>
+  </si>
+  <si>
+    <t>https://i.imgur.gg/ERjWTfe-IMG_20260705_174054.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/yykLghU-IMG_20260705_174152.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/dcsEDNF-IMG_20260705_173922.jpg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2001,6 +2007,14 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -2040,16 +2054,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2615,7 +2632,7 @@
       <c r="I2">
         <v>1</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="2" t="s">
         <v>133</v>
       </c>
       <c r="K2" t="s">
@@ -3473,6 +3490,9 @@
       <sortCondition ref="B1"/>
     </sortState>
   </autoFilter>
+  <hyperlinks>
+    <hyperlink ref="J2" r:id="rId1" xr:uid="{D12460E6-324C-456F-A9D4-16EEC3C8BCA4}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
@@ -3512,933 +3532,933 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>149</v>
+        <v>296</v>
       </c>
       <c r="B2" t="s">
-        <v>129</v>
+        <v>101</v>
       </c>
       <c r="C2" t="s">
-        <v>133</v>
+        <v>297</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F2" t="s">
-        <v>150</v>
+        <v>287</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>151</v>
+        <v>290</v>
       </c>
       <c r="B3" t="s">
-        <v>129</v>
+        <v>101</v>
       </c>
       <c r="C3" t="s">
-        <v>152</v>
+        <v>291</v>
       </c>
       <c r="D3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" t="s">
-        <v>150</v>
+        <v>287</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>154</v>
+        <v>286</v>
       </c>
       <c r="B4" t="s">
-        <v>129</v>
+        <v>101</v>
       </c>
       <c r="C4" t="s">
-        <v>155</v>
+        <v>106</v>
       </c>
       <c r="D4" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="E4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F4" t="s">
-        <v>150</v>
+        <v>287</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>156</v>
+        <v>288</v>
       </c>
       <c r="B5" t="s">
-        <v>129</v>
+        <v>101</v>
       </c>
       <c r="C5" t="s">
-        <v>155</v>
+        <v>289</v>
       </c>
       <c r="D5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>150</v>
+        <v>287</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>157</v>
+        <v>292</v>
       </c>
       <c r="B6" t="s">
-        <v>129</v>
+        <v>101</v>
       </c>
       <c r="C6" t="s">
-        <v>158</v>
+        <v>293</v>
       </c>
       <c r="D6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F6" t="s">
-        <v>150</v>
+        <v>287</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>159</v>
+        <v>294</v>
       </c>
       <c r="B7" t="s">
-        <v>129</v>
+        <v>101</v>
       </c>
       <c r="C7" t="s">
-        <v>160</v>
+        <v>295</v>
       </c>
       <c r="D7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F7" t="s">
-        <v>150</v>
+        <v>287</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>161</v>
+        <v>310</v>
       </c>
       <c r="B8" t="s">
-        <v>129</v>
+        <v>112</v>
       </c>
       <c r="C8" t="s">
-        <v>162</v>
+        <v>311</v>
       </c>
       <c r="D8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E8">
         <v>6</v>
       </c>
       <c r="F8" t="s">
-        <v>150</v>
+        <v>299</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>163</v>
+        <v>304</v>
       </c>
       <c r="B9" t="s">
-        <v>69</v>
+        <v>112</v>
       </c>
       <c r="C9" t="s">
-        <v>164</v>
+        <v>305</v>
       </c>
       <c r="D9" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>165</v>
+        <v>299</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>166</v>
+        <v>306</v>
       </c>
       <c r="B10" t="s">
-        <v>69</v>
+        <v>112</v>
       </c>
       <c r="C10" t="s">
-        <v>167</v>
+        <v>307</v>
       </c>
       <c r="D10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F10" t="s">
-        <v>165</v>
+        <v>299</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>168</v>
+        <v>302</v>
       </c>
       <c r="B11" t="s">
-        <v>69</v>
+        <v>112</v>
       </c>
       <c r="C11" t="s">
-        <v>169</v>
+        <v>303</v>
       </c>
       <c r="D11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E11">
         <v>2</v>
       </c>
       <c r="F11" t="s">
-        <v>165</v>
+        <v>299</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>170</v>
+        <v>308</v>
       </c>
       <c r="B12" t="s">
-        <v>69</v>
+        <v>112</v>
       </c>
       <c r="C12" t="s">
-        <v>171</v>
+        <v>309</v>
       </c>
       <c r="D12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E12">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F12" t="s">
-        <v>165</v>
+        <v>299</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>172</v>
+        <v>300</v>
       </c>
       <c r="B13" t="s">
-        <v>69</v>
+        <v>112</v>
       </c>
       <c r="C13" t="s">
-        <v>173</v>
+        <v>301</v>
       </c>
       <c r="D13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E13">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>165</v>
+        <v>299</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>174</v>
+        <v>298</v>
       </c>
       <c r="B14" t="s">
-        <v>69</v>
+        <v>112</v>
       </c>
       <c r="C14" t="s">
-        <v>175</v>
+        <v>116</v>
       </c>
       <c r="D14" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="E14">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F14" t="s">
-        <v>165</v>
+        <v>299</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>176</v>
+        <v>402</v>
       </c>
       <c r="B15" t="s">
-        <v>69</v>
+        <v>124</v>
       </c>
       <c r="C15" t="s">
-        <v>177</v>
+        <v>128</v>
       </c>
       <c r="D15" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="E15">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F15" t="s">
-        <v>165</v>
+        <v>403</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>178</v>
+        <v>410</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>124</v>
       </c>
       <c r="C16" t="s">
-        <v>179</v>
+        <v>411</v>
       </c>
       <c r="D16" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E16">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F16" t="s">
-        <v>165</v>
+        <v>403</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>180</v>
+        <v>416</v>
       </c>
       <c r="B17" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="C17" t="s">
-        <v>145</v>
+        <v>417</v>
       </c>
       <c r="D17" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E17">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F17" t="s">
-        <v>181</v>
+        <v>403</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>182</v>
+        <v>412</v>
       </c>
       <c r="B18" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="C18" t="s">
-        <v>183</v>
+        <v>413</v>
       </c>
       <c r="D18" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E18">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F18" t="s">
-        <v>181</v>
+        <v>403</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>184</v>
+        <v>408</v>
       </c>
       <c r="B19" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="C19" t="s">
-        <v>185</v>
+        <v>409</v>
       </c>
       <c r="D19" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E19">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F19" t="s">
-        <v>181</v>
+        <v>403</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>186</v>
+        <v>406</v>
       </c>
       <c r="B20" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="C20" t="s">
-        <v>187</v>
+        <v>407</v>
       </c>
       <c r="D20" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E20">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F20" t="s">
-        <v>181</v>
+        <v>403</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>188</v>
+        <v>404</v>
       </c>
       <c r="B21" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="C21" t="s">
-        <v>189</v>
+        <v>405</v>
       </c>
       <c r="D21" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E21">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>181</v>
+        <v>403</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>190</v>
+        <v>414</v>
       </c>
       <c r="B22" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="C22" t="s">
-        <v>191</v>
+        <v>415</v>
       </c>
       <c r="D22" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F22" t="s">
-        <v>181</v>
+        <v>403</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>192</v>
+        <v>334</v>
       </c>
       <c r="B23" t="s">
-        <v>141</v>
+        <v>85</v>
       </c>
       <c r="C23" t="s">
-        <v>193</v>
+        <v>90</v>
       </c>
       <c r="D23" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="E23">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F23" t="s">
-        <v>181</v>
+        <v>335</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>194</v>
+        <v>336</v>
       </c>
       <c r="B24" t="s">
-        <v>141</v>
+        <v>85</v>
       </c>
       <c r="C24" t="s">
-        <v>195</v>
+        <v>337</v>
       </c>
       <c r="D24" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E24">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>181</v>
+        <v>335</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>196</v>
+        <v>340</v>
       </c>
       <c r="B25" t="s">
-        <v>141</v>
+        <v>85</v>
       </c>
       <c r="C25" t="s">
-        <v>197</v>
+        <v>341</v>
       </c>
       <c r="D25" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E25">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F25" t="s">
-        <v>181</v>
+        <v>335</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>198</v>
+        <v>342</v>
       </c>
       <c r="B26" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="C26" t="s">
-        <v>80</v>
+        <v>343</v>
       </c>
       <c r="D26" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E26">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F26" t="s">
-        <v>199</v>
+        <v>335</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>200</v>
+        <v>338</v>
       </c>
       <c r="B27" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="C27" t="s">
-        <v>201</v>
+        <v>339</v>
       </c>
       <c r="D27" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F27" t="s">
-        <v>199</v>
+        <v>335</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>202</v>
+        <v>344</v>
       </c>
       <c r="B28" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="C28" t="s">
-        <v>203</v>
+        <v>345</v>
       </c>
       <c r="D28" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E28">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F28" t="s">
-        <v>199</v>
+        <v>335</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>204</v>
+        <v>392</v>
       </c>
       <c r="B29" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="C29" t="s">
-        <v>205</v>
+        <v>393</v>
       </c>
       <c r="D29" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E29">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F29" t="s">
-        <v>199</v>
+        <v>381</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>206</v>
+        <v>386</v>
       </c>
       <c r="B30" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="C30" t="s">
-        <v>207</v>
+        <v>387</v>
       </c>
       <c r="D30" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E30">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F30" t="s">
-        <v>199</v>
+        <v>381</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>208</v>
+        <v>382</v>
       </c>
       <c r="B31" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="C31" t="s">
-        <v>209</v>
+        <v>383</v>
       </c>
       <c r="D31" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E31">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F31" t="s">
-        <v>199</v>
+        <v>381</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>210</v>
+        <v>384</v>
       </c>
       <c r="B32" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="C32" t="s">
-        <v>211</v>
+        <v>385</v>
       </c>
       <c r="D32" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E32">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F32" t="s">
-        <v>199</v>
+        <v>381</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>212</v>
+        <v>390</v>
       </c>
       <c r="B33" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="C33" t="s">
-        <v>111</v>
+        <v>391</v>
       </c>
       <c r="D33" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E33">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F33" t="s">
-        <v>213</v>
+        <v>381</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>214</v>
+        <v>398</v>
       </c>
       <c r="B34" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="C34" t="s">
-        <v>215</v>
+        <v>399</v>
       </c>
       <c r="D34" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E34">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F34" t="s">
-        <v>213</v>
+        <v>381</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>216</v>
+        <v>396</v>
       </c>
       <c r="B35" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="C35" t="s">
-        <v>217</v>
+        <v>397</v>
       </c>
       <c r="D35" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E35">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F35" t="s">
-        <v>213</v>
+        <v>381</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>218</v>
+        <v>388</v>
       </c>
       <c r="B36" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="C36" t="s">
-        <v>219</v>
+        <v>389</v>
       </c>
       <c r="D36" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F36" t="s">
-        <v>213</v>
+        <v>381</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>220</v>
+        <v>380</v>
       </c>
       <c r="B37" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="C37" t="s">
-        <v>221</v>
+        <v>100</v>
       </c>
       <c r="D37" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="E37">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F37" t="s">
-        <v>213</v>
+        <v>381</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>222</v>
+        <v>394</v>
       </c>
       <c r="B38" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="C38" t="s">
-        <v>223</v>
+        <v>395</v>
       </c>
       <c r="D38" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E38">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F38" t="s">
-        <v>213</v>
+        <v>381</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
-        <v>224</v>
+        <v>400</v>
       </c>
       <c r="B39" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="C39" t="s">
-        <v>225</v>
+        <v>401</v>
       </c>
       <c r="D39" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E39">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F39" t="s">
-        <v>213</v>
+        <v>381</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
+        <v>233</v>
+      </c>
+      <c r="B40" t="s">
+        <v>62</v>
+      </c>
+      <c r="C40" t="s">
+        <v>234</v>
+      </c>
+      <c r="D40" t="s">
+        <v>152</v>
+      </c>
+      <c r="E40">
+        <v>4</v>
+      </c>
+      <c r="F40" t="s">
         <v>226</v>
-      </c>
-      <c r="B40" t="s">
-        <v>107</v>
-      </c>
-      <c r="C40" t="s">
-        <v>227</v>
-      </c>
-      <c r="D40" t="s">
-        <v>153</v>
-      </c>
-      <c r="E40">
-        <v>7</v>
-      </c>
-      <c r="F40" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="B41" t="s">
         <v>62</v>
       </c>
       <c r="C41" t="s">
-        <v>68</v>
+        <v>238</v>
       </c>
       <c r="D41" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E41">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F41" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="B42" t="s">
         <v>62</v>
       </c>
       <c r="C42" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="D42" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E42">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F42" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B43" t="s">
         <v>62</v>
       </c>
       <c r="C43" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D43" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E43">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F43" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B44" t="s">
         <v>62</v>
       </c>
       <c r="C44" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="D44" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E44">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F44" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="B45" t="s">
         <v>62</v>
       </c>
       <c r="C45" t="s">
-        <v>237</v>
+        <v>68</v>
       </c>
       <c r="D45" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="E45">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F45" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="B46" t="s">
         <v>62</v>
       </c>
       <c r="C46" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="D46" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E46">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F46" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
-        <v>240</v>
+        <v>326</v>
       </c>
       <c r="B47" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="C47" t="s">
-        <v>241</v>
+        <v>327</v>
       </c>
       <c r="D47" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E47">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F47" t="s">
-        <v>229</v>
+        <v>323</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
-        <v>242</v>
+        <v>322</v>
       </c>
       <c r="B48" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="C48" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="D48" t="s">
         <v>10</v>
@@ -4447,598 +4467,598 @@
         <v>0</v>
       </c>
       <c r="F48" t="s">
-        <v>243</v>
+        <v>323</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
-        <v>244</v>
+        <v>330</v>
       </c>
       <c r="B49" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="C49" t="s">
-        <v>245</v>
+        <v>331</v>
       </c>
       <c r="D49" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E49">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F49" t="s">
-        <v>243</v>
+        <v>323</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
-        <v>246</v>
+        <v>328</v>
       </c>
       <c r="B50" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="C50" t="s">
-        <v>247</v>
+        <v>329</v>
       </c>
       <c r="D50" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E50">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F50" t="s">
-        <v>243</v>
+        <v>323</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
-        <v>248</v>
+        <v>324</v>
       </c>
       <c r="B51" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="C51" t="s">
-        <v>249</v>
+        <v>325</v>
       </c>
       <c r="D51" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E51">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F51" t="s">
-        <v>243</v>
+        <v>323</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
-        <v>250</v>
+        <v>332</v>
       </c>
       <c r="B52" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="C52" t="s">
-        <v>251</v>
+        <v>333</v>
       </c>
       <c r="D52" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E52">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F52" t="s">
-        <v>243</v>
+        <v>323</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
-        <v>252</v>
+        <v>316</v>
       </c>
       <c r="B53" t="s">
-        <v>27</v>
+        <v>81</v>
       </c>
       <c r="C53" t="s">
-        <v>253</v>
+        <v>317</v>
       </c>
       <c r="D53" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E53">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F53" t="s">
-        <v>243</v>
+        <v>313</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
-        <v>254</v>
+        <v>318</v>
       </c>
       <c r="B54" t="s">
-        <v>27</v>
+        <v>81</v>
       </c>
       <c r="C54" t="s">
-        <v>255</v>
+        <v>319</v>
       </c>
       <c r="D54" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E54">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F54" t="s">
-        <v>243</v>
+        <v>313</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
-        <v>256</v>
+        <v>314</v>
       </c>
       <c r="B55" t="s">
-        <v>27</v>
+        <v>81</v>
       </c>
       <c r="C55" t="s">
-        <v>257</v>
+        <v>315</v>
       </c>
       <c r="D55" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E55">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F55" t="s">
-        <v>243</v>
+        <v>313</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
-        <v>258</v>
+        <v>320</v>
       </c>
       <c r="B56" t="s">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="C56" t="s">
-        <v>41</v>
+        <v>321</v>
       </c>
       <c r="D56" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E56">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F56" t="s">
-        <v>259</v>
+        <v>313</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
-        <v>260</v>
+        <v>312</v>
       </c>
       <c r="B57" t="s">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="C57" t="s">
-        <v>261</v>
+        <v>84</v>
       </c>
       <c r="D57" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="E57">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F57" t="s">
-        <v>259</v>
+        <v>313</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
-        <v>262</v>
+        <v>156</v>
       </c>
       <c r="B58" t="s">
-        <v>35</v>
+        <v>129</v>
       </c>
       <c r="C58" t="s">
-        <v>263</v>
+        <v>133</v>
       </c>
       <c r="D58" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E58">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F58" t="s">
-        <v>259</v>
+        <v>150</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
-        <v>264</v>
+        <v>155</v>
       </c>
       <c r="B59" t="s">
-        <v>35</v>
+        <v>129</v>
       </c>
       <c r="C59" t="s">
-        <v>265</v>
+        <v>538</v>
       </c>
       <c r="D59" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E59">
         <v>3</v>
       </c>
       <c r="F59" t="s">
-        <v>259</v>
+        <v>150</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
-        <v>266</v>
+        <v>149</v>
       </c>
       <c r="B60" t="s">
-        <v>35</v>
+        <v>129</v>
       </c>
       <c r="C60" t="s">
-        <v>267</v>
+        <v>154</v>
       </c>
       <c r="D60" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="E60">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F60" t="s">
-        <v>259</v>
+        <v>150</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
-        <v>268</v>
+        <v>151</v>
       </c>
       <c r="B61" t="s">
-        <v>35</v>
+        <v>129</v>
       </c>
       <c r="C61" t="s">
-        <v>267</v>
+        <v>539</v>
       </c>
       <c r="D61" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E61">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F61" t="s">
-        <v>259</v>
+        <v>150</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
-        <v>269</v>
+        <v>153</v>
       </c>
       <c r="B62" t="s">
-        <v>35</v>
+        <v>129</v>
       </c>
       <c r="C62" t="s">
-        <v>270</v>
+        <v>540</v>
       </c>
       <c r="D62" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E62">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F62" t="s">
-        <v>259</v>
+        <v>150</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
-        <v>271</v>
+        <v>157</v>
       </c>
       <c r="B63" t="s">
-        <v>35</v>
+        <v>129</v>
       </c>
       <c r="C63" t="s">
-        <v>272</v>
+        <v>158</v>
       </c>
       <c r="D63" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E63">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F63" t="s">
-        <v>259</v>
+        <v>150</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
-        <v>273</v>
+        <v>159</v>
       </c>
       <c r="B64" t="s">
-        <v>43</v>
+        <v>129</v>
       </c>
       <c r="C64" t="s">
-        <v>47</v>
+        <v>541</v>
       </c>
       <c r="D64" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E64">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F64" t="s">
-        <v>274</v>
+        <v>150</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
-        <v>275</v>
+        <v>346</v>
       </c>
       <c r="B65" t="s">
-        <v>43</v>
+        <v>91</v>
       </c>
       <c r="C65" t="s">
-        <v>276</v>
+        <v>95</v>
       </c>
       <c r="D65" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="E65">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F65" t="s">
-        <v>274</v>
+        <v>347</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
-        <v>277</v>
+        <v>350</v>
       </c>
       <c r="B66" t="s">
-        <v>43</v>
+        <v>91</v>
       </c>
       <c r="C66" t="s">
-        <v>278</v>
+        <v>351</v>
       </c>
       <c r="D66" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E66">
         <v>2</v>
       </c>
       <c r="F66" t="s">
-        <v>274</v>
+        <v>347</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
-        <v>279</v>
+        <v>354</v>
       </c>
       <c r="B67" t="s">
-        <v>43</v>
+        <v>91</v>
       </c>
       <c r="C67" t="s">
-        <v>280</v>
+        <v>355</v>
       </c>
       <c r="D67" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E67">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F67" t="s">
-        <v>274</v>
+        <v>347</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
-        <v>281</v>
+        <v>356</v>
       </c>
       <c r="B68" t="s">
-        <v>43</v>
+        <v>91</v>
       </c>
       <c r="C68" t="s">
-        <v>282</v>
+        <v>357</v>
       </c>
       <c r="D68" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E68">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F68" t="s">
-        <v>274</v>
+        <v>347</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
-        <v>283</v>
+        <v>352</v>
       </c>
       <c r="B69" t="s">
-        <v>43</v>
+        <v>91</v>
       </c>
       <c r="C69" t="s">
-        <v>284</v>
+        <v>353</v>
       </c>
       <c r="D69" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E69">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F69" t="s">
-        <v>274</v>
+        <v>347</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
-        <v>285</v>
+        <v>348</v>
       </c>
       <c r="B70" t="s">
-        <v>43</v>
+        <v>91</v>
       </c>
       <c r="C70" t="s">
-        <v>286</v>
+        <v>349</v>
       </c>
       <c r="D70" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E70">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F70" t="s">
-        <v>274</v>
+        <v>347</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
-        <v>287</v>
+        <v>175</v>
       </c>
       <c r="B71" t="s">
-        <v>43</v>
+        <v>69</v>
       </c>
       <c r="C71" t="s">
-        <v>288</v>
+        <v>176</v>
       </c>
       <c r="D71" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E71">
         <v>7</v>
       </c>
       <c r="F71" t="s">
-        <v>274</v>
+        <v>162</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
-        <v>289</v>
+        <v>167</v>
       </c>
       <c r="B72" t="s">
-        <v>101</v>
+        <v>69</v>
       </c>
       <c r="C72" t="s">
-        <v>106</v>
+        <v>168</v>
       </c>
       <c r="D72" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E72">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F72" t="s">
-        <v>290</v>
+        <v>162</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
-        <v>291</v>
+        <v>169</v>
       </c>
       <c r="B73" t="s">
-        <v>101</v>
+        <v>69</v>
       </c>
       <c r="C73" t="s">
-        <v>292</v>
+        <v>170</v>
       </c>
       <c r="D73" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E73">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F73" t="s">
-        <v>290</v>
+        <v>162</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
-        <v>293</v>
+        <v>171</v>
       </c>
       <c r="B74" t="s">
-        <v>101</v>
+        <v>69</v>
       </c>
       <c r="C74" t="s">
-        <v>294</v>
+        <v>172</v>
       </c>
       <c r="D74" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E74">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F74" t="s">
-        <v>290</v>
+        <v>162</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
-        <v>295</v>
+        <v>173</v>
       </c>
       <c r="B75" t="s">
-        <v>101</v>
+        <v>69</v>
       </c>
       <c r="C75" t="s">
-        <v>296</v>
+        <v>174</v>
       </c>
       <c r="D75" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E75">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F75" t="s">
-        <v>290</v>
+        <v>162</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
-        <v>297</v>
+        <v>165</v>
       </c>
       <c r="B76" t="s">
-        <v>101</v>
+        <v>69</v>
       </c>
       <c r="C76" t="s">
-        <v>298</v>
+        <v>166</v>
       </c>
       <c r="D76" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E76">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F76" t="s">
-        <v>290</v>
+        <v>162</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
-        <v>299</v>
+        <v>163</v>
       </c>
       <c r="B77" t="s">
-        <v>101</v>
+        <v>69</v>
       </c>
       <c r="C77" t="s">
-        <v>300</v>
+        <v>164</v>
       </c>
       <c r="D77" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E77">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F77" t="s">
-        <v>290</v>
+        <v>162</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
-        <v>301</v>
+        <v>160</v>
       </c>
       <c r="B78" t="s">
-        <v>112</v>
+        <v>69</v>
       </c>
       <c r="C78" t="s">
-        <v>116</v>
+        <v>161</v>
       </c>
       <c r="D78" t="s">
         <v>10</v>
@@ -5047,238 +5067,238 @@
         <v>0</v>
       </c>
       <c r="F78" t="s">
-        <v>302</v>
+        <v>162</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
-        <v>303</v>
+        <v>201</v>
       </c>
       <c r="B79" t="s">
-        <v>112</v>
+        <v>76</v>
       </c>
       <c r="C79" t="s">
-        <v>304</v>
+        <v>202</v>
       </c>
       <c r="D79" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E79">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F79" t="s">
-        <v>302</v>
+        <v>196</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
-        <v>305</v>
+        <v>205</v>
       </c>
       <c r="B80" t="s">
-        <v>112</v>
+        <v>76</v>
       </c>
       <c r="C80" t="s">
-        <v>306</v>
+        <v>206</v>
       </c>
       <c r="D80" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="E80">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F80" t="s">
-        <v>302</v>
+        <v>196</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
-        <v>307</v>
+        <v>199</v>
       </c>
       <c r="B81" t="s">
-        <v>112</v>
+        <v>76</v>
       </c>
       <c r="C81" t="s">
-        <v>308</v>
+        <v>200</v>
       </c>
       <c r="D81" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E81">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F81" t="s">
-        <v>302</v>
+        <v>196</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
-        <v>309</v>
+        <v>207</v>
       </c>
       <c r="B82" t="s">
-        <v>112</v>
+        <v>76</v>
       </c>
       <c r="C82" t="s">
-        <v>310</v>
+        <v>208</v>
       </c>
       <c r="D82" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E82">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F82" t="s">
-        <v>302</v>
+        <v>196</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
-        <v>311</v>
+        <v>195</v>
       </c>
       <c r="B83" t="s">
-        <v>112</v>
+        <v>76</v>
       </c>
       <c r="C83" t="s">
-        <v>312</v>
+        <v>80</v>
       </c>
       <c r="D83" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E83">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F83" t="s">
-        <v>302</v>
+        <v>196</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
-        <v>313</v>
+        <v>203</v>
       </c>
       <c r="B84" t="s">
-        <v>112</v>
+        <v>76</v>
       </c>
       <c r="C84" t="s">
-        <v>314</v>
+        <v>204</v>
       </c>
       <c r="D84" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E84">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F84" t="s">
-        <v>302</v>
+        <v>196</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
-        <v>315</v>
+        <v>197</v>
       </c>
       <c r="B85" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C85" t="s">
-        <v>84</v>
+        <v>198</v>
       </c>
       <c r="D85" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E85">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F85" t="s">
-        <v>316</v>
+        <v>196</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
-        <v>317</v>
+        <v>360</v>
       </c>
       <c r="B86" t="s">
-        <v>81</v>
+        <v>56</v>
       </c>
       <c r="C86" t="s">
-        <v>318</v>
+        <v>361</v>
       </c>
       <c r="D86" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E86">
         <v>1</v>
       </c>
       <c r="F86" t="s">
-        <v>316</v>
+        <v>359</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
-        <v>319</v>
+        <v>370</v>
       </c>
       <c r="B87" t="s">
-        <v>81</v>
+        <v>56</v>
       </c>
       <c r="C87" t="s">
-        <v>320</v>
+        <v>371</v>
       </c>
       <c r="D87" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E87">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F87" t="s">
-        <v>316</v>
+        <v>359</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
-        <v>321</v>
+        <v>362</v>
       </c>
       <c r="B88" t="s">
-        <v>81</v>
+        <v>56</v>
       </c>
       <c r="C88" t="s">
-        <v>322</v>
+        <v>363</v>
       </c>
       <c r="D88" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E88">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F88" t="s">
-        <v>316</v>
+        <v>359</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
-        <v>323</v>
+        <v>368</v>
       </c>
       <c r="B89" t="s">
-        <v>81</v>
+        <v>56</v>
       </c>
       <c r="C89" t="s">
-        <v>324</v>
+        <v>369</v>
       </c>
       <c r="D89" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E89">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F89" t="s">
-        <v>316</v>
+        <v>359</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
-        <v>325</v>
+        <v>358</v>
       </c>
       <c r="B90" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="C90" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="D90" t="s">
         <v>10</v>
@@ -5287,1251 +5307,1261 @@
         <v>0</v>
       </c>
       <c r="F90" t="s">
-        <v>326</v>
+        <v>359</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
-        <v>327</v>
+        <v>374</v>
       </c>
       <c r="B91" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="C91" t="s">
-        <v>328</v>
+        <v>375</v>
       </c>
       <c r="D91" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E91">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F91" t="s">
-        <v>326</v>
+        <v>359</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
-        <v>329</v>
+        <v>364</v>
       </c>
       <c r="B92" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="C92" t="s">
-        <v>330</v>
+        <v>365</v>
       </c>
       <c r="D92" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E92">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F92" t="s">
-        <v>326</v>
+        <v>359</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
-        <v>331</v>
+        <v>378</v>
       </c>
       <c r="B93" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="C93" t="s">
-        <v>332</v>
+        <v>379</v>
       </c>
       <c r="D93" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E93">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F93" t="s">
-        <v>326</v>
+        <v>359</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A94" t="s">
-        <v>333</v>
+        <v>366</v>
       </c>
       <c r="B94" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="C94" t="s">
-        <v>334</v>
+        <v>367</v>
       </c>
       <c r="D94" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E94">
         <v>4</v>
       </c>
       <c r="F94" t="s">
-        <v>326</v>
+        <v>359</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A95" t="s">
-        <v>335</v>
+        <v>372</v>
       </c>
       <c r="B95" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="C95" t="s">
-        <v>336</v>
+        <v>373</v>
       </c>
       <c r="D95" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E95">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F95" t="s">
-        <v>326</v>
+        <v>359</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
-        <v>337</v>
+        <v>376</v>
       </c>
       <c r="B96" t="s">
-        <v>85</v>
+        <v>56</v>
       </c>
       <c r="C96" t="s">
-        <v>90</v>
+        <v>377</v>
       </c>
       <c r="D96" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E96">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F96" t="s">
-        <v>338</v>
+        <v>359</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
-        <v>339</v>
+        <v>428</v>
       </c>
       <c r="B97" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="C97" t="s">
-        <v>340</v>
+        <v>429</v>
       </c>
       <c r="D97" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E97">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F97" t="s">
-        <v>338</v>
+        <v>419</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
-        <v>341</v>
+        <v>422</v>
       </c>
       <c r="B98" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="C98" t="s">
-        <v>342</v>
+        <v>423</v>
       </c>
       <c r="D98" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E98">
         <v>2</v>
       </c>
       <c r="F98" t="s">
-        <v>338</v>
+        <v>419</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A99" t="s">
-        <v>343</v>
+        <v>424</v>
       </c>
       <c r="B99" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="C99" t="s">
-        <v>344</v>
+        <v>425</v>
       </c>
       <c r="D99" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E99">
         <v>3</v>
       </c>
       <c r="F99" t="s">
-        <v>338</v>
+        <v>419</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A100" t="s">
-        <v>345</v>
+        <v>426</v>
       </c>
       <c r="B100" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="C100" t="s">
-        <v>346</v>
+        <v>427</v>
       </c>
       <c r="D100" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E100">
         <v>4</v>
       </c>
       <c r="F100" t="s">
-        <v>338</v>
+        <v>419</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A101" t="s">
-        <v>347</v>
+        <v>418</v>
       </c>
       <c r="B101" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="C101" t="s">
-        <v>348</v>
+        <v>123</v>
       </c>
       <c r="D101" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="E101">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F101" t="s">
-        <v>338</v>
+        <v>419</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A102" t="s">
-        <v>349</v>
+        <v>430</v>
       </c>
       <c r="B102" t="s">
-        <v>91</v>
+        <v>117</v>
       </c>
       <c r="C102" t="s">
-        <v>95</v>
+        <v>431</v>
       </c>
       <c r="D102" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E102">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F102" t="s">
-        <v>350</v>
+        <v>419</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A103" t="s">
-        <v>351</v>
+        <v>420</v>
       </c>
       <c r="B103" t="s">
-        <v>91</v>
+        <v>117</v>
       </c>
       <c r="C103" t="s">
-        <v>352</v>
+        <v>421</v>
       </c>
       <c r="D103" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E103">
         <v>1</v>
       </c>
       <c r="F103" t="s">
-        <v>350</v>
+        <v>419</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A104" t="s">
-        <v>353</v>
+        <v>249</v>
       </c>
       <c r="B104" t="s">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="C104" t="s">
-        <v>354</v>
+        <v>250</v>
       </c>
       <c r="D104" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E104">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F104" t="s">
-        <v>350</v>
+        <v>240</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A105" t="s">
-        <v>355</v>
+        <v>243</v>
       </c>
       <c r="B105" t="s">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="C105" t="s">
-        <v>356</v>
+        <v>244</v>
       </c>
       <c r="D105" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E105">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F105" t="s">
-        <v>350</v>
+        <v>240</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A106" t="s">
-        <v>357</v>
+        <v>245</v>
       </c>
       <c r="B106" t="s">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="C106" t="s">
-        <v>358</v>
+        <v>246</v>
       </c>
       <c r="D106" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E106">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F106" t="s">
-        <v>350</v>
+        <v>240</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A107" t="s">
-        <v>359</v>
+        <v>251</v>
       </c>
       <c r="B107" t="s">
-        <v>91</v>
+        <v>27</v>
       </c>
       <c r="C107" t="s">
-        <v>360</v>
+        <v>252</v>
       </c>
       <c r="D107" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E107">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F107" t="s">
-        <v>350</v>
+        <v>240</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A108" t="s">
-        <v>361</v>
+        <v>241</v>
       </c>
       <c r="B108" t="s">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="C108" t="s">
-        <v>61</v>
+        <v>242</v>
       </c>
       <c r="D108" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E108">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F108" t="s">
-        <v>362</v>
+        <v>240</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A109" t="s">
-        <v>363</v>
+        <v>247</v>
       </c>
       <c r="B109" t="s">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="C109" t="s">
-        <v>364</v>
+        <v>248</v>
       </c>
       <c r="D109" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E109">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F109" t="s">
-        <v>362</v>
+        <v>240</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A110" t="s">
-        <v>365</v>
+        <v>253</v>
       </c>
       <c r="B110" t="s">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="C110" t="s">
-        <v>366</v>
+        <v>254</v>
       </c>
       <c r="D110" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E110">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F110" t="s">
-        <v>362</v>
+        <v>240</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A111" t="s">
-        <v>367</v>
+        <v>239</v>
       </c>
       <c r="B111" t="s">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="C111" t="s">
-        <v>368</v>
+        <v>33</v>
       </c>
       <c r="D111" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="E111">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F111" t="s">
-        <v>362</v>
+        <v>240</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A112" t="s">
-        <v>369</v>
+        <v>213</v>
       </c>
       <c r="B112" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="C112" t="s">
-        <v>370</v>
+        <v>214</v>
       </c>
       <c r="D112" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E112">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F112" t="s">
-        <v>362</v>
+        <v>210</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A113" t="s">
-        <v>371</v>
+        <v>223</v>
       </c>
       <c r="B113" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="C113" t="s">
-        <v>372</v>
+        <v>224</v>
       </c>
       <c r="D113" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E113">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F113" t="s">
-        <v>362</v>
+        <v>210</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A114" t="s">
-        <v>373</v>
+        <v>209</v>
       </c>
       <c r="B114" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="C114" t="s">
-        <v>374</v>
+        <v>111</v>
       </c>
       <c r="D114" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="E114">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F114" t="s">
-        <v>362</v>
+        <v>210</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A115" t="s">
-        <v>375</v>
+        <v>211</v>
       </c>
       <c r="B115" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="C115" t="s">
-        <v>376</v>
+        <v>212</v>
       </c>
       <c r="D115" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E115">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F115" t="s">
-        <v>362</v>
+        <v>210</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A116" t="s">
-        <v>377</v>
+        <v>217</v>
       </c>
       <c r="B116" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="C116" t="s">
-        <v>378</v>
+        <v>218</v>
       </c>
       <c r="D116" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E116">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F116" t="s">
-        <v>362</v>
+        <v>210</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A117" t="s">
-        <v>379</v>
+        <v>219</v>
       </c>
       <c r="B117" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="C117" t="s">
-        <v>380</v>
+        <v>220</v>
       </c>
       <c r="D117" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E117">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F117" t="s">
-        <v>362</v>
+        <v>210</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A118" t="s">
-        <v>381</v>
+        <v>221</v>
       </c>
       <c r="B118" t="s">
-        <v>56</v>
+        <v>107</v>
       </c>
       <c r="C118" t="s">
-        <v>382</v>
+        <v>222</v>
       </c>
       <c r="D118" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E118">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F118" t="s">
-        <v>362</v>
+        <v>210</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A119" t="s">
-        <v>383</v>
+        <v>215</v>
       </c>
       <c r="B119" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="C119" t="s">
-        <v>100</v>
+        <v>216</v>
       </c>
       <c r="D119" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E119">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F119" t="s">
-        <v>384</v>
+        <v>210</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A120" t="s">
-        <v>385</v>
+        <v>282</v>
       </c>
       <c r="B120" t="s">
-        <v>96</v>
+        <v>43</v>
       </c>
       <c r="C120" t="s">
-        <v>386</v>
+        <v>283</v>
       </c>
       <c r="D120" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E120">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F120" t="s">
-        <v>384</v>
+        <v>271</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A121" t="s">
-        <v>387</v>
+        <v>278</v>
       </c>
       <c r="B121" t="s">
-        <v>96</v>
+        <v>43</v>
       </c>
       <c r="C121" t="s">
-        <v>388</v>
+        <v>279</v>
       </c>
       <c r="D121" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E121">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F121" t="s">
-        <v>384</v>
+        <v>271</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A122" t="s">
-        <v>389</v>
+        <v>276</v>
       </c>
       <c r="B122" t="s">
-        <v>96</v>
+        <v>43</v>
       </c>
       <c r="C122" t="s">
-        <v>390</v>
+        <v>277</v>
       </c>
       <c r="D122" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E122">
         <v>3</v>
       </c>
       <c r="F122" t="s">
-        <v>384</v>
+        <v>271</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A123" t="s">
-        <v>391</v>
+        <v>280</v>
       </c>
       <c r="B123" t="s">
-        <v>96</v>
+        <v>43</v>
       </c>
       <c r="C123" t="s">
-        <v>392</v>
+        <v>281</v>
       </c>
       <c r="D123" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E123">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F123" t="s">
-        <v>384</v>
+        <v>271</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A124" t="s">
-        <v>393</v>
+        <v>272</v>
       </c>
       <c r="B124" t="s">
-        <v>96</v>
+        <v>43</v>
       </c>
       <c r="C124" t="s">
-        <v>394</v>
+        <v>273</v>
       </c>
       <c r="D124" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E124">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F124" t="s">
-        <v>384</v>
+        <v>271</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A125" t="s">
-        <v>395</v>
+        <v>284</v>
       </c>
       <c r="B125" t="s">
-        <v>96</v>
+        <v>43</v>
       </c>
       <c r="C125" t="s">
-        <v>396</v>
+        <v>285</v>
       </c>
       <c r="D125" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E125">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F125" t="s">
-        <v>384</v>
+        <v>271</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A126" t="s">
-        <v>397</v>
+        <v>274</v>
       </c>
       <c r="B126" t="s">
-        <v>96</v>
+        <v>43</v>
       </c>
       <c r="C126" t="s">
-        <v>398</v>
+        <v>275</v>
       </c>
       <c r="D126" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E126">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F126" t="s">
-        <v>384</v>
+        <v>271</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A127" t="s">
-        <v>399</v>
+        <v>270</v>
       </c>
       <c r="B127" t="s">
-        <v>96</v>
+        <v>43</v>
       </c>
       <c r="C127" t="s">
-        <v>400</v>
+        <v>47</v>
       </c>
       <c r="D127" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="E127">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F127" t="s">
-        <v>384</v>
+        <v>271</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A128" t="s">
-        <v>401</v>
+        <v>446</v>
       </c>
       <c r="B128" t="s">
-        <v>96</v>
+        <v>134</v>
       </c>
       <c r="C128" t="s">
-        <v>402</v>
+        <v>447</v>
       </c>
       <c r="D128" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E128">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F128" t="s">
-        <v>384</v>
+        <v>433</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A129" t="s">
-        <v>403</v>
+        <v>444</v>
       </c>
       <c r="B129" t="s">
-        <v>96</v>
+        <v>134</v>
       </c>
       <c r="C129" t="s">
-        <v>404</v>
+        <v>445</v>
       </c>
       <c r="D129" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E129">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F129" t="s">
-        <v>384</v>
+        <v>433</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A130" t="s">
-        <v>405</v>
+        <v>434</v>
       </c>
       <c r="B130" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="C130" t="s">
-        <v>128</v>
+        <v>435</v>
       </c>
       <c r="D130" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E130">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F130" t="s">
-        <v>406</v>
+        <v>433</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A131" t="s">
-        <v>407</v>
+        <v>432</v>
       </c>
       <c r="B131" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="C131" t="s">
-        <v>408</v>
+        <v>140</v>
       </c>
       <c r="D131" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="E131">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F131" t="s">
-        <v>406</v>
+        <v>433</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A132" t="s">
-        <v>409</v>
+        <v>438</v>
       </c>
       <c r="B132" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="C132" t="s">
-        <v>410</v>
+        <v>439</v>
       </c>
       <c r="D132" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E132">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F132" t="s">
-        <v>406</v>
+        <v>433</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A133" t="s">
-        <v>411</v>
+        <v>442</v>
       </c>
       <c r="B133" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="C133" t="s">
-        <v>412</v>
+        <v>443</v>
       </c>
       <c r="D133" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E133">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F133" t="s">
-        <v>406</v>
+        <v>433</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A134" t="s">
-        <v>413</v>
+        <v>436</v>
       </c>
       <c r="B134" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="C134" t="s">
-        <v>414</v>
+        <v>437</v>
       </c>
       <c r="D134" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E134">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F134" t="s">
-        <v>406</v>
+        <v>433</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A135" t="s">
-        <v>415</v>
+        <v>440</v>
       </c>
       <c r="B135" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="C135" t="s">
-        <v>416</v>
+        <v>441</v>
       </c>
       <c r="D135" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E135">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F135" t="s">
-        <v>406</v>
+        <v>433</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A136" t="s">
-        <v>417</v>
+        <v>187</v>
       </c>
       <c r="B136" t="s">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="C136" t="s">
-        <v>418</v>
+        <v>188</v>
       </c>
       <c r="D136" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E136">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F136" t="s">
-        <v>406</v>
+        <v>178</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A137" t="s">
-        <v>419</v>
+        <v>191</v>
       </c>
       <c r="B137" t="s">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="C137" t="s">
-        <v>420</v>
+        <v>192</v>
       </c>
       <c r="D137" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E137">
         <v>7</v>
       </c>
       <c r="F137" t="s">
-        <v>406</v>
+        <v>178</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A138" t="s">
-        <v>421</v>
+        <v>193</v>
       </c>
       <c r="B138" t="s">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="C138" t="s">
-        <v>123</v>
+        <v>194</v>
       </c>
       <c r="D138" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E138">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F138" t="s">
-        <v>422</v>
+        <v>178</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A139" t="s">
-        <v>423</v>
+        <v>181</v>
       </c>
       <c r="B139" t="s">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="C139" t="s">
-        <v>424</v>
+        <v>182</v>
       </c>
       <c r="D139" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E139">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F139" t="s">
-        <v>422</v>
+        <v>178</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A140" t="s">
-        <v>425</v>
+        <v>179</v>
       </c>
       <c r="B140" t="s">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="C140" t="s">
-        <v>426</v>
+        <v>180</v>
       </c>
       <c r="D140" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E140">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F140" t="s">
-        <v>422</v>
+        <v>178</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A141" t="s">
-        <v>427</v>
+        <v>177</v>
       </c>
       <c r="B141" t="s">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="C141" t="s">
-        <v>428</v>
+        <v>145</v>
       </c>
       <c r="D141" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="E141">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F141" t="s">
-        <v>422</v>
+        <v>178</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A142" t="s">
-        <v>429</v>
+        <v>183</v>
       </c>
       <c r="B142" t="s">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="C142" t="s">
-        <v>430</v>
+        <v>184</v>
       </c>
       <c r="D142" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E142">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F142" t="s">
-        <v>422</v>
+        <v>178</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A143" t="s">
-        <v>431</v>
+        <v>185</v>
       </c>
       <c r="B143" t="s">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="C143" t="s">
-        <v>432</v>
+        <v>186</v>
       </c>
       <c r="D143" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E143">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F143" t="s">
-        <v>422</v>
+        <v>178</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A144" t="s">
-        <v>433</v>
+        <v>189</v>
       </c>
       <c r="B144" t="s">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="C144" t="s">
-        <v>434</v>
+        <v>190</v>
       </c>
       <c r="D144" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E144">
         <v>6</v>
       </c>
       <c r="F144" t="s">
-        <v>422</v>
+        <v>178</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A145" t="s">
-        <v>435</v>
+        <v>266</v>
       </c>
       <c r="B145" t="s">
-        <v>134</v>
+        <v>35</v>
       </c>
       <c r="C145" t="s">
-        <v>140</v>
+        <v>267</v>
       </c>
       <c r="D145" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E145">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F145" t="s">
-        <v>436</v>
+        <v>256</v>
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A146" t="s">
-        <v>437</v>
+        <v>261</v>
       </c>
       <c r="B146" t="s">
-        <v>134</v>
+        <v>35</v>
       </c>
       <c r="C146" t="s">
-        <v>438</v>
+        <v>262</v>
       </c>
       <c r="D146" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E146">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F146" t="s">
-        <v>436</v>
+        <v>256</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A147" t="s">
-        <v>439</v>
+        <v>257</v>
       </c>
       <c r="B147" t="s">
-        <v>134</v>
+        <v>35</v>
       </c>
       <c r="C147" t="s">
-        <v>440</v>
+        <v>258</v>
       </c>
       <c r="D147" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E147">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F147" t="s">
-        <v>436</v>
+        <v>256</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A148" t="s">
-        <v>441</v>
+        <v>263</v>
       </c>
       <c r="B148" t="s">
-        <v>134</v>
+        <v>35</v>
       </c>
       <c r="C148" t="s">
-        <v>442</v>
+        <v>264</v>
       </c>
       <c r="D148" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E148">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F148" t="s">
-        <v>436</v>
+        <v>256</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A149" t="s">
-        <v>443</v>
+        <v>268</v>
       </c>
       <c r="B149" t="s">
-        <v>134</v>
+        <v>35</v>
       </c>
       <c r="C149" t="s">
-        <v>444</v>
+        <v>269</v>
       </c>
       <c r="D149" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E149">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F149" t="s">
-        <v>436</v>
+        <v>256</v>
       </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A150" t="s">
-        <v>445</v>
+        <v>255</v>
       </c>
       <c r="B150" t="s">
-        <v>134</v>
+        <v>35</v>
       </c>
       <c r="C150" t="s">
-        <v>446</v>
+        <v>41</v>
       </c>
       <c r="D150" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="E150">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F150" t="s">
-        <v>436</v>
+        <v>256</v>
       </c>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A151" t="s">
-        <v>447</v>
+        <v>265</v>
       </c>
       <c r="B151" t="s">
-        <v>134</v>
+        <v>35</v>
       </c>
       <c r="C151" t="s">
-        <v>448</v>
+        <v>264</v>
       </c>
       <c r="D151" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E151">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F151" t="s">
-        <v>436</v>
+        <v>256</v>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A152" t="s">
-        <v>449</v>
+        <v>259</v>
       </c>
       <c r="B152" t="s">
-        <v>134</v>
+        <v>35</v>
       </c>
       <c r="C152" t="s">
-        <v>450</v>
+        <v>260</v>
       </c>
       <c r="D152" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E152">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F152" t="s">
-        <v>436</v>
+        <v>256</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <autoFilter ref="A1:F1" xr:uid="{00000000-0009-0000-0000-000002000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F152">
+      <sortCondition ref="B1"/>
+    </sortState>
+  </autoFilter>
+  <hyperlinks>
+    <hyperlink ref="C58" r:id="rId1" xr:uid="{108D5BAC-872E-4FA1-9AA5-5DD2A9B28BDD}"/>
+    <hyperlink ref="C60" r:id="rId2" xr:uid="{2C3D556D-39AA-4885-AD25-D636D5148266}"/>
+    <hyperlink ref="C61" r:id="rId3" xr:uid="{8AA99DC7-365F-46C5-809B-E7D4E69A9EDF}"/>
+    <hyperlink ref="C63" r:id="rId4" xr:uid="{368E5479-408D-4DE9-814B-B19BEA995149}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
@@ -6564,58 +6594,58 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>453</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>454</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>458</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>459</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>460</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>461</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>462</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>463</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>465</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>466</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>467</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>468</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>6</v>
@@ -6626,61 +6656,61 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
+        <v>506</v>
+      </c>
+      <c r="B2" t="s">
+        <v>507</v>
+      </c>
+      <c r="C2" t="s">
+        <v>508</v>
+      </c>
+      <c r="D2" t="s">
         <v>509</v>
       </c>
-      <c r="B2" t="s">
+      <c r="E2" t="s">
         <v>510</v>
       </c>
-      <c r="C2" t="s">
+      <c r="F2" t="s">
         <v>511</v>
       </c>
-      <c r="D2" t="s">
+      <c r="G2" t="s">
         <v>512</v>
       </c>
-      <c r="E2" t="s">
+      <c r="H2" t="s">
         <v>513</v>
       </c>
-      <c r="F2" t="s">
+      <c r="I2" t="s">
         <v>514</v>
       </c>
-      <c r="G2" t="s">
+      <c r="J2" t="s">
         <v>515</v>
       </c>
-      <c r="H2" t="s">
+      <c r="K2" t="s">
         <v>516</v>
       </c>
-      <c r="I2" t="s">
+      <c r="L2" t="s">
         <v>517</v>
       </c>
-      <c r="J2" t="s">
+      <c r="M2" t="s">
         <v>518</v>
-      </c>
-      <c r="K2" t="s">
-        <v>519</v>
-      </c>
-      <c r="L2" t="s">
-        <v>520</v>
-      </c>
-      <c r="M2" t="s">
-        <v>521</v>
       </c>
       <c r="N2" t="s">
         <v>138</v>
       </c>
       <c r="O2" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="P2" t="s">
         <v>139</v>
       </c>
       <c r="Q2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="T2" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="U2" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
     </row>
   </sheetData>
@@ -6709,22 +6739,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>146</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>6</v>
@@ -6732,13 +6762,13 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="B2" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="C2" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="D2" t="s">
         <v>136</v>
@@ -6750,7 +6780,7 @@
         <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
     </row>
   </sheetData>
@@ -6777,16 +6807,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>6</v>
@@ -6794,70 +6824,70 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="B2" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="C2" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="D2" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="E2" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
+        <v>528</v>
+      </c>
+      <c r="B3" t="s">
+        <v>506</v>
+      </c>
+      <c r="C3" t="s">
+        <v>529</v>
+      </c>
+      <c r="D3" t="s">
+        <v>530</v>
+      </c>
+      <c r="E3" t="s">
         <v>531</v>
-      </c>
-      <c r="B3" t="s">
-        <v>509</v>
-      </c>
-      <c r="C3" t="s">
-        <v>532</v>
-      </c>
-      <c r="D3" t="s">
-        <v>533</v>
-      </c>
-      <c r="E3" t="s">
-        <v>534</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
+        <v>532</v>
+      </c>
+      <c r="B4" t="s">
+        <v>506</v>
+      </c>
+      <c r="C4" t="s">
+        <v>533</v>
+      </c>
+      <c r="D4" t="s">
+        <v>534</v>
+      </c>
+      <c r="E4" t="s">
         <v>535</v>
-      </c>
-      <c r="B4" t="s">
-        <v>509</v>
-      </c>
-      <c r="C4" t="s">
-        <v>536</v>
-      </c>
-      <c r="D4" t="s">
-        <v>537</v>
-      </c>
-      <c r="E4" t="s">
-        <v>538</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="B5" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="C5" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="D5" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="E5" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
     </row>
   </sheetData>
@@ -6885,19 +6915,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>6</v>
@@ -6908,22 +6938,22 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
+        <v>475</v>
+      </c>
+      <c r="B2" t="s">
+        <v>476</v>
+      </c>
+      <c r="C2" t="s">
+        <v>477</v>
+      </c>
+      <c r="D2" t="s">
         <v>478</v>
-      </c>
-      <c r="B2" t="s">
-        <v>479</v>
-      </c>
-      <c r="C2" t="s">
-        <v>480</v>
-      </c>
-      <c r="D2" t="s">
-        <v>481</v>
       </c>
       <c r="E2" t="s">
         <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="G2" t="s">
         <v>11</v>
@@ -6951,18 +6981,18 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -6973,7 +7003,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="B3">
         <v>4</v>
@@ -6984,7 +7014,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -6995,7 +7025,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -7006,233 +7036,233 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B6" t="s">
         <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B7" t="s">
         <v>35</v>
       </c>
       <c r="C7" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B8" t="s">
         <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B9" t="s">
         <v>48</v>
       </c>
       <c r="C9" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B10" t="s">
         <v>56</v>
       </c>
       <c r="C10" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B11" t="s">
         <v>62</v>
       </c>
       <c r="C11" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B12" t="s">
         <v>69</v>
       </c>
       <c r="C12" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B13" t="s">
         <v>76</v>
       </c>
       <c r="C13" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B14" t="s">
         <v>81</v>
       </c>
       <c r="C14" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B15" t="s">
         <v>85</v>
       </c>
       <c r="C15" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B16" t="s">
         <v>91</v>
       </c>
       <c r="C16" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B17" t="s">
         <v>96</v>
       </c>
       <c r="C17" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B18" t="s">
         <v>101</v>
       </c>
       <c r="C18" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B19" t="s">
         <v>107</v>
       </c>
       <c r="C19" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B20" t="s">
         <v>112</v>
       </c>
       <c r="C20" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B21" t="s">
         <v>117</v>
       </c>
       <c r="C21" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B22" t="s">
         <v>124</v>
       </c>
       <c r="C22" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B23" t="s">
         <v>129</v>
       </c>
       <c r="C23" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B24" t="s">
         <v>134</v>
       </c>
       <c r="C24" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B25" t="s">
         <v>141</v>
       </c>
       <c r="C25" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="B26" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="C26" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Update seed data and improve image handling in product generation
</commit_message>
<xml_diff>
--- a/chinni-treasure/exports/chinni-treasure-export-2026-07-18T18-45-09.xlsx
+++ b/chinni-treasure/exports/chinni-treasure-export-2026-07-18T18-45-09.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{817BC37A-6F29-40F1-82BA-DC9129D204D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{569311F6-2F09-4DC1-8EB5-A1641E9E89B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2895" yWindow="1868" windowWidth="16200" windowHeight="9307" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
@@ -17,12 +17,15 @@
     <sheet name="Admins" sheetId="7" r:id="rId7"/>
     <sheet name="ID Lookup" sheetId="8" r:id="rId8"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Product Images'!$A$1:$F$152</definedName>
+  </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="542">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="543">
   <si>
     <t>ID</t>
   </si>
@@ -853,15 +856,9 @@
     <t>d2419bf7-54a9-4508-9dd2-1059b5142163</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/asnOI23-IMG_20260705_163534.jpg</t>
-  </si>
-  <si>
     <t>ad367dca-c393-4307-9731-29ced6e2f759</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/TbMHSBd-IMG_20260705_163729.jpg</t>
-  </si>
-  <si>
     <t>82b38006-f0de-46bb-9c3a-295945fef6b7</t>
   </si>
   <si>
@@ -871,21 +868,12 @@
     <t>9147991d-d1ee-42f3-8479-0208a7b4c4c8</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/uMICzTw-IMG_20260705_163602.jpg</t>
-  </si>
-  <si>
     <t>99e29e94-f86b-428c-a6af-3dc26b4dad36</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/CaSUkND-IMG_20260705_163606.jpg</t>
-  </si>
-  <si>
     <t>a43110d5-8581-4bb7-b90e-4fac35e95a95</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/2prDVur-IMG_20260705_163620.jpg</t>
-  </si>
-  <si>
     <t>332372fb-9bef-43d9-8e06-bf33eeb4f5af</t>
   </si>
   <si>
@@ -901,15 +889,9 @@
     <t>e10244f0-ed7e-40cd-bb0b-b2a94552a50b</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/gPhThze-IMG_20260705_155515.jpg</t>
-  </si>
-  <si>
     <t>d654169b-445e-4102-9433-efbf4a72eaab</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/POeQ3vJ-IMG_20260705_155729.jpg</t>
-  </si>
-  <si>
     <t>f3557160-16ef-41bb-b07f-d9e605be66f4</t>
   </si>
   <si>
@@ -925,9 +907,6 @@
     <t>74357b3d-953f-4e29-bac4-765b0e849dad</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/H8if62Z-WhatsApp_Image_2026-07-05_at_8.23.28_PM_(1).jpeg</t>
-  </si>
-  <si>
     <t>fbaf6ab0-760f-4f7e-ab56-059e04cddbaa</t>
   </si>
   <si>
@@ -961,21 +940,12 @@
     <t>8675ecc0-a3b0-431d-98ef-81c907bf4a1e</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/y7bKdkd-IMG_20260705_170706.jpg</t>
-  </si>
-  <si>
     <t>20191ed9-5ecc-4222-acda-14537907b72c</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/Fcae0PT-IMG_20260705_170717.jpg</t>
-  </si>
-  <si>
     <t>e68bf781-3af1-4f7b-9224-8630439867be</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/6Dk9y30-IMG_20260705_170727.jpg</t>
-  </si>
-  <si>
     <t>7ca97743-1297-47bf-bcf7-4a7473fb7bd7</t>
   </si>
   <si>
@@ -985,9 +955,6 @@
     <t>b4fb0af1-7c91-4db6-91d8-7579c885e4fc</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/Pca7Qx0-IMG_20260705_170818.jpg</t>
-  </si>
-  <si>
     <t>3e6d5814-cc09-4d24-9c20-fc0097d8ceba</t>
   </si>
   <si>
@@ -997,27 +964,15 @@
     <t>56b09a6f-519b-4180-bc85-a475cf602efb</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/MpnlvKu-IMG_20260705_164715.jpg</t>
-  </si>
-  <si>
     <t>05f5cd5a-b922-41ad-a6d6-bc44182240c1</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/XEcEMCr-IMG_20260705_171521.jpg</t>
-  </si>
-  <si>
     <t>ed135245-35af-4386-9290-b1a6f1f5cc9a</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/7hHNIn9-IMG_20260705_171539.jpg</t>
-  </si>
-  <si>
     <t>90cde30c-5532-4fa8-83ea-8fa51da4ba7e</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/9DIwgl3-IMG_20260705_171554.jpg</t>
-  </si>
-  <si>
     <t>ad9f98cd-b728-4fad-8d2b-486978b77507</t>
   </si>
   <si>
@@ -1045,13 +1000,7 @@
     <t>b32bf5c7-152e-43ed-9a18-ea9cf929b968</t>
   </si>
   <si>
-    <t>https://i.imgur.gg/XBAU5Wz-IMG_20260705_172242.jpg</t>
-  </si>
-  <si>
     <t>f6d81e18-a2a7-427c-b99d-40cc0a03ca84</t>
-  </si>
-  <si>
-    <t>https://i.imgur.gg/NpSLdpF-IMG_20260705_172314.jpg</t>
   </si>
   <si>
     <t>af4bdf26-a389-48ea-a119-750550594b67</t>
@@ -1988,6 +1937,82 @@
   <si>
     <t xml:space="preserve">
 https://i.imgur.gg/dcsEDNF-IMG_20260705_173922.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/asnOI23-IMG_20260705_163534.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/TbMHSBd-IMG_20260705_163729.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/uMICzTw-IMG_20260705_163602.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/CaSUkND-IMG_20260705_163606.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/2prDVur-IMG_20260705_163620.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/eggPVAF-IMG_20260703_111828.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/gPhThze-IMG_20260705_155515.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/POeQ3vJ-IMG_20260705_155729.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/ExV2tjL-IMG_20260705_170653.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/y7bKdkd-IMG_20260705_170706.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/Fcae0PT-IMG_20260705_170717.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/6Dk9y30-IMG_20260705_170727.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/MpnlvKu-IMG_20260705_164715.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/XEcEMCr-IMG_20260705_171521.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/7hHNIn9-IMG_20260705_171539.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/9DIwgl3-IMG_20260705_171554.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/ISUicHP-IMG_20260705_164031.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/XBAU5Wz-IMG_20260705_172242.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://i.imgur.gg/NpSLdpF-IMG_20260705_172314.jpg</t>
   </si>
 </sst>
 </file>
@@ -2009,12 +2034,11 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <u/>
+      <b/>
       <sz val="11"/>
-      <color theme="10"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -2054,19 +2078,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2444,16 +2468,16 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F2" t="s">
         <v>10</v>
@@ -2467,16 +2491,16 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3" t="s">
         <v>10</v>
@@ -2513,16 +2537,16 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F5" t="s">
         <v>10</v>
@@ -2535,7 +2559,11 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:H1" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H5">
+      <sortCondition ref="A1"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
@@ -2632,7 +2660,7 @@
       <c r="I2">
         <v>1</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" t="s">
         <v>133</v>
       </c>
       <c r="K2" t="s">
@@ -3492,6 +3520,13 @@
   </autoFilter>
   <hyperlinks>
     <hyperlink ref="J2" r:id="rId1" xr:uid="{D12460E6-324C-456F-A9D4-16EEC3C8BCA4}"/>
+    <hyperlink ref="J4" r:id="rId2" xr:uid="{2EDD8AD0-6436-4539-9B14-D6A6746E1353}"/>
+    <hyperlink ref="J5" r:id="rId3" xr:uid="{656DC348-CFC6-4B18-BA25-9CE8B99C5C81}"/>
+    <hyperlink ref="J6" r:id="rId4" xr:uid="{7D162952-5CB2-4B3D-96A0-C3F5C45D7737}"/>
+    <hyperlink ref="J7" r:id="rId5" xr:uid="{59884DF2-5301-4642-A585-40B0C45F6D81}"/>
+    <hyperlink ref="J8" r:id="rId6" xr:uid="{DABF14E4-6403-437F-AFE0-BB3758B14D2A}"/>
+    <hyperlink ref="J9" r:id="rId7" xr:uid="{5F09AE0A-1014-44EB-97C2-C10A3C747BCA}"/>
+    <hyperlink ref="J10" r:id="rId8" xr:uid="{5A7CE844-401E-461E-936D-4163E9B55837}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
@@ -3514,7 +3549,7 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>146</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -3532,267 +3567,267 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>296</v>
+        <v>268</v>
       </c>
       <c r="B2" t="s">
         <v>101</v>
       </c>
       <c r="C2" t="s">
-        <v>297</v>
+        <v>106</v>
       </c>
       <c r="D2" t="s">
-        <v>152</v>
+        <v>10</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>287</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>290</v>
+        <v>270</v>
       </c>
       <c r="B3" t="s">
         <v>101</v>
       </c>
       <c r="C3" t="s">
-        <v>291</v>
+        <v>271</v>
       </c>
       <c r="D3" t="s">
         <v>152</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>287</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>286</v>
+        <v>272</v>
       </c>
       <c r="B4" t="s">
         <v>101</v>
       </c>
       <c r="C4" t="s">
-        <v>106</v>
+        <v>273</v>
       </c>
       <c r="D4" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F4" t="s">
-        <v>287</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>288</v>
+        <v>274</v>
       </c>
       <c r="B5" t="s">
         <v>101</v>
       </c>
       <c r="C5" t="s">
-        <v>289</v>
+        <v>275</v>
       </c>
       <c r="D5" t="s">
         <v>152</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F5" t="s">
-        <v>287</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>292</v>
+        <v>276</v>
       </c>
       <c r="B6" t="s">
         <v>101</v>
       </c>
       <c r="C6" t="s">
-        <v>293</v>
+        <v>277</v>
       </c>
       <c r="D6" t="s">
         <v>152</v>
       </c>
       <c r="E6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F6" t="s">
-        <v>287</v>
+        <v>269</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>294</v>
+        <v>278</v>
       </c>
       <c r="B7" t="s">
         <v>101</v>
       </c>
       <c r="C7" t="s">
-        <v>295</v>
+        <v>279</v>
       </c>
       <c r="D7" t="s">
         <v>152</v>
       </c>
       <c r="E7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F7" t="s">
-        <v>287</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>310</v>
+        <v>280</v>
       </c>
       <c r="B8" t="s">
         <v>112</v>
       </c>
       <c r="C8" t="s">
-        <v>311</v>
+        <v>116</v>
       </c>
       <c r="D8" t="s">
-        <v>152</v>
+        <v>10</v>
       </c>
       <c r="E8">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F8" t="s">
-        <v>299</v>
+        <v>281</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>304</v>
+        <v>282</v>
       </c>
       <c r="B9" t="s">
         <v>112</v>
       </c>
       <c r="C9" t="s">
-        <v>305</v>
+        <v>283</v>
       </c>
       <c r="D9" t="s">
         <v>152</v>
       </c>
       <c r="E9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>299</v>
+        <v>281</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>306</v>
+        <v>284</v>
       </c>
       <c r="B10" t="s">
         <v>112</v>
       </c>
       <c r="C10" t="s">
-        <v>307</v>
+        <v>285</v>
       </c>
       <c r="D10" t="s">
         <v>152</v>
       </c>
       <c r="E10">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F10" t="s">
-        <v>299</v>
+        <v>281</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>302</v>
+        <v>286</v>
       </c>
       <c r="B11" t="s">
         <v>112</v>
       </c>
       <c r="C11" t="s">
-        <v>303</v>
+        <v>287</v>
       </c>
       <c r="D11" t="s">
         <v>152</v>
       </c>
       <c r="E11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" t="s">
-        <v>299</v>
+        <v>281</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>308</v>
+        <v>288</v>
       </c>
       <c r="B12" t="s">
         <v>112</v>
       </c>
       <c r="C12" t="s">
-        <v>309</v>
+        <v>289</v>
       </c>
       <c r="D12" t="s">
         <v>152</v>
       </c>
       <c r="E12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F12" t="s">
-        <v>299</v>
+        <v>281</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="B13" t="s">
         <v>112</v>
       </c>
       <c r="C13" t="s">
-        <v>301</v>
+        <v>291</v>
       </c>
       <c r="D13" t="s">
         <v>152</v>
       </c>
       <c r="E13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F13" t="s">
-        <v>299</v>
+        <v>281</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="B14" t="s">
         <v>112</v>
       </c>
       <c r="C14" t="s">
-        <v>116</v>
+        <v>293</v>
       </c>
       <c r="D14" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F14" t="s">
-        <v>299</v>
+        <v>281</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>402</v>
+        <v>384</v>
       </c>
       <c r="B15" t="s">
         <v>124</v>
@@ -3807,18 +3842,18 @@
         <v>0</v>
       </c>
       <c r="F15" t="s">
-        <v>403</v>
+        <v>385</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>410</v>
+        <v>392</v>
       </c>
       <c r="B16" t="s">
         <v>124</v>
       </c>
       <c r="C16" t="s">
-        <v>411</v>
+        <v>393</v>
       </c>
       <c r="D16" t="s">
         <v>152</v>
@@ -3827,18 +3862,18 @@
         <v>4</v>
       </c>
       <c r="F16" t="s">
-        <v>403</v>
+        <v>385</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>416</v>
+        <v>398</v>
       </c>
       <c r="B17" t="s">
         <v>124</v>
       </c>
       <c r="C17" t="s">
-        <v>417</v>
+        <v>399</v>
       </c>
       <c r="D17" t="s">
         <v>152</v>
@@ -3847,18 +3882,18 @@
         <v>7</v>
       </c>
       <c r="F17" t="s">
-        <v>403</v>
+        <v>385</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>412</v>
+        <v>394</v>
       </c>
       <c r="B18" t="s">
         <v>124</v>
       </c>
       <c r="C18" t="s">
-        <v>413</v>
+        <v>395</v>
       </c>
       <c r="D18" t="s">
         <v>152</v>
@@ -3867,18 +3902,18 @@
         <v>5</v>
       </c>
       <c r="F18" t="s">
-        <v>403</v>
+        <v>385</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>408</v>
+        <v>390</v>
       </c>
       <c r="B19" t="s">
         <v>124</v>
       </c>
       <c r="C19" t="s">
-        <v>409</v>
+        <v>391</v>
       </c>
       <c r="D19" t="s">
         <v>152</v>
@@ -3887,18 +3922,18 @@
         <v>3</v>
       </c>
       <c r="F19" t="s">
-        <v>403</v>
+        <v>385</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>406</v>
+        <v>388</v>
       </c>
       <c r="B20" t="s">
         <v>124</v>
       </c>
       <c r="C20" t="s">
-        <v>407</v>
+        <v>389</v>
       </c>
       <c r="D20" t="s">
         <v>152</v>
@@ -3907,18 +3942,18 @@
         <v>2</v>
       </c>
       <c r="F20" t="s">
-        <v>403</v>
+        <v>385</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>404</v>
+        <v>386</v>
       </c>
       <c r="B21" t="s">
         <v>124</v>
       </c>
       <c r="C21" t="s">
-        <v>405</v>
+        <v>387</v>
       </c>
       <c r="D21" t="s">
         <v>152</v>
@@ -3927,18 +3962,18 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>403</v>
+        <v>385</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>414</v>
+        <v>396</v>
       </c>
       <c r="B22" t="s">
         <v>124</v>
       </c>
       <c r="C22" t="s">
-        <v>415</v>
+        <v>397</v>
       </c>
       <c r="D22" t="s">
         <v>152</v>
@@ -3947,12 +3982,12 @@
         <v>6</v>
       </c>
       <c r="F22" t="s">
-        <v>403</v>
+        <v>385</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>334</v>
+        <v>316</v>
       </c>
       <c r="B23" t="s">
         <v>85</v>
@@ -3967,18 +4002,18 @@
         <v>0</v>
       </c>
       <c r="F23" t="s">
-        <v>335</v>
+        <v>317</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>336</v>
+        <v>318</v>
       </c>
       <c r="B24" t="s">
         <v>85</v>
       </c>
       <c r="C24" t="s">
-        <v>337</v>
+        <v>319</v>
       </c>
       <c r="D24" t="s">
         <v>152</v>
@@ -3987,18 +4022,18 @@
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>335</v>
+        <v>317</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>340</v>
+        <v>322</v>
       </c>
       <c r="B25" t="s">
         <v>85</v>
       </c>
       <c r="C25" t="s">
-        <v>341</v>
+        <v>323</v>
       </c>
       <c r="D25" t="s">
         <v>152</v>
@@ -4007,18 +4042,18 @@
         <v>3</v>
       </c>
       <c r="F25" t="s">
-        <v>335</v>
+        <v>317</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>342</v>
+        <v>324</v>
       </c>
       <c r="B26" t="s">
         <v>85</v>
       </c>
       <c r="C26" t="s">
-        <v>343</v>
+        <v>325</v>
       </c>
       <c r="D26" t="s">
         <v>152</v>
@@ -4027,18 +4062,18 @@
         <v>4</v>
       </c>
       <c r="F26" t="s">
-        <v>335</v>
+        <v>317</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>338</v>
+        <v>320</v>
       </c>
       <c r="B27" t="s">
         <v>85</v>
       </c>
       <c r="C27" t="s">
-        <v>339</v>
+        <v>321</v>
       </c>
       <c r="D27" t="s">
         <v>152</v>
@@ -4047,18 +4082,18 @@
         <v>2</v>
       </c>
       <c r="F27" t="s">
-        <v>335</v>
+        <v>317</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>344</v>
+        <v>326</v>
       </c>
       <c r="B28" t="s">
         <v>85</v>
       </c>
       <c r="C28" t="s">
-        <v>345</v>
+        <v>327</v>
       </c>
       <c r="D28" t="s">
         <v>152</v>
@@ -4067,18 +4102,18 @@
         <v>5</v>
       </c>
       <c r="F28" t="s">
-        <v>335</v>
+        <v>317</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>392</v>
+        <v>374</v>
       </c>
       <c r="B29" t="s">
         <v>96</v>
       </c>
       <c r="C29" t="s">
-        <v>393</v>
+        <v>375</v>
       </c>
       <c r="D29" t="s">
         <v>152</v>
@@ -4087,18 +4122,18 @@
         <v>6</v>
       </c>
       <c r="F29" t="s">
-        <v>381</v>
+        <v>363</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>386</v>
+        <v>368</v>
       </c>
       <c r="B30" t="s">
         <v>96</v>
       </c>
       <c r="C30" t="s">
-        <v>387</v>
+        <v>369</v>
       </c>
       <c r="D30" t="s">
         <v>152</v>
@@ -4107,18 +4142,18 @@
         <v>3</v>
       </c>
       <c r="F30" t="s">
-        <v>381</v>
+        <v>363</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>382</v>
+        <v>364</v>
       </c>
       <c r="B31" t="s">
         <v>96</v>
       </c>
       <c r="C31" t="s">
-        <v>383</v>
+        <v>365</v>
       </c>
       <c r="D31" t="s">
         <v>152</v>
@@ -4127,18 +4162,18 @@
         <v>1</v>
       </c>
       <c r="F31" t="s">
-        <v>381</v>
+        <v>363</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>384</v>
+        <v>366</v>
       </c>
       <c r="B32" t="s">
         <v>96</v>
       </c>
       <c r="C32" t="s">
-        <v>385</v>
+        <v>367</v>
       </c>
       <c r="D32" t="s">
         <v>152</v>
@@ -4147,18 +4182,18 @@
         <v>2</v>
       </c>
       <c r="F32" t="s">
-        <v>381</v>
+        <v>363</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>390</v>
+        <v>372</v>
       </c>
       <c r="B33" t="s">
         <v>96</v>
       </c>
       <c r="C33" t="s">
-        <v>391</v>
+        <v>373</v>
       </c>
       <c r="D33" t="s">
         <v>152</v>
@@ -4167,18 +4202,18 @@
         <v>5</v>
       </c>
       <c r="F33" t="s">
-        <v>381</v>
+        <v>363</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>398</v>
+        <v>380</v>
       </c>
       <c r="B34" t="s">
         <v>96</v>
       </c>
       <c r="C34" t="s">
-        <v>399</v>
+        <v>381</v>
       </c>
       <c r="D34" t="s">
         <v>152</v>
@@ -4187,18 +4222,18 @@
         <v>9</v>
       </c>
       <c r="F34" t="s">
-        <v>381</v>
+        <v>363</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>396</v>
+        <v>378</v>
       </c>
       <c r="B35" t="s">
         <v>96</v>
       </c>
       <c r="C35" t="s">
-        <v>397</v>
+        <v>379</v>
       </c>
       <c r="D35" t="s">
         <v>152</v>
@@ -4207,18 +4242,18 @@
         <v>8</v>
       </c>
       <c r="F35" t="s">
-        <v>381</v>
+        <v>363</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>388</v>
+        <v>370</v>
       </c>
       <c r="B36" t="s">
         <v>96</v>
       </c>
       <c r="C36" t="s">
-        <v>389</v>
+        <v>371</v>
       </c>
       <c r="D36" t="s">
         <v>152</v>
@@ -4227,12 +4262,12 @@
         <v>4</v>
       </c>
       <c r="F36" t="s">
-        <v>381</v>
+        <v>363</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>380</v>
+        <v>362</v>
       </c>
       <c r="B37" t="s">
         <v>96</v>
@@ -4247,18 +4282,18 @@
         <v>0</v>
       </c>
       <c r="F37" t="s">
-        <v>381</v>
+        <v>363</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>394</v>
+        <v>376</v>
       </c>
       <c r="B38" t="s">
         <v>96</v>
       </c>
       <c r="C38" t="s">
-        <v>395</v>
+        <v>377</v>
       </c>
       <c r="D38" t="s">
         <v>152</v>
@@ -4267,18 +4302,18 @@
         <v>7</v>
       </c>
       <c r="F38" t="s">
-        <v>381</v>
+        <v>363</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
-        <v>400</v>
+        <v>382</v>
       </c>
       <c r="B39" t="s">
         <v>96</v>
       </c>
       <c r="C39" t="s">
-        <v>401</v>
+        <v>383</v>
       </c>
       <c r="D39" t="s">
         <v>152</v>
@@ -4287,78 +4322,78 @@
         <v>10</v>
       </c>
       <c r="F39" t="s">
-        <v>381</v>
+        <v>363</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
-        <v>233</v>
+        <v>209</v>
       </c>
       <c r="B40" t="s">
         <v>62</v>
       </c>
       <c r="C40" t="s">
-        <v>234</v>
+        <v>540</v>
       </c>
       <c r="D40" t="s">
-        <v>152</v>
+        <v>10</v>
       </c>
       <c r="E40">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F40" t="s">
-        <v>226</v>
+        <v>210</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
-        <v>237</v>
+        <v>211</v>
       </c>
       <c r="B41" t="s">
         <v>62</v>
       </c>
       <c r="C41" t="s">
-        <v>238</v>
+        <v>541</v>
       </c>
       <c r="D41" t="s">
         <v>152</v>
       </c>
       <c r="E41">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F41" t="s">
-        <v>226</v>
+        <v>210</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
-        <v>235</v>
+        <v>212</v>
       </c>
       <c r="B42" t="s">
         <v>62</v>
       </c>
       <c r="C42" t="s">
-        <v>236</v>
+        <v>542</v>
       </c>
       <c r="D42" t="s">
         <v>152</v>
       </c>
       <c r="E42">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F42" t="s">
-        <v>226</v>
+        <v>210</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
-        <v>231</v>
+        <v>213</v>
       </c>
       <c r="B43" t="s">
         <v>62</v>
       </c>
       <c r="C43" t="s">
-        <v>232</v>
+        <v>214</v>
       </c>
       <c r="D43" t="s">
         <v>152</v>
@@ -4367,78 +4402,78 @@
         <v>3</v>
       </c>
       <c r="F43" t="s">
-        <v>226</v>
+        <v>210</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="B44" t="s">
         <v>62</v>
       </c>
       <c r="C44" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="D44" t="s">
         <v>152</v>
       </c>
       <c r="E44">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F44" t="s">
-        <v>226</v>
+        <v>210</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="B45" t="s">
         <v>62</v>
       </c>
       <c r="C45" t="s">
-        <v>68</v>
+        <v>218</v>
       </c>
       <c r="D45" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E45">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F45" t="s">
-        <v>226</v>
+        <v>210</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
-        <v>229</v>
+        <v>219</v>
       </c>
       <c r="B46" t="s">
         <v>62</v>
       </c>
       <c r="C46" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="D46" t="s">
         <v>152</v>
       </c>
       <c r="E46">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F46" t="s">
-        <v>226</v>
+        <v>210</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
-        <v>326</v>
+        <v>308</v>
       </c>
       <c r="B47" t="s">
         <v>48</v>
       </c>
       <c r="C47" t="s">
-        <v>327</v>
+        <v>309</v>
       </c>
       <c r="D47" t="s">
         <v>152</v>
@@ -4447,12 +4482,12 @@
         <v>2</v>
       </c>
       <c r="F47" t="s">
-        <v>323</v>
+        <v>305</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
-        <v>322</v>
+        <v>304</v>
       </c>
       <c r="B48" t="s">
         <v>48</v>
@@ -4467,18 +4502,18 @@
         <v>0</v>
       </c>
       <c r="F48" t="s">
-        <v>323</v>
+        <v>305</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
-        <v>330</v>
+        <v>312</v>
       </c>
       <c r="B49" t="s">
         <v>48</v>
       </c>
       <c r="C49" t="s">
-        <v>331</v>
+        <v>313</v>
       </c>
       <c r="D49" t="s">
         <v>152</v>
@@ -4487,18 +4522,18 @@
         <v>4</v>
       </c>
       <c r="F49" t="s">
-        <v>323</v>
+        <v>305</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
-        <v>328</v>
+        <v>310</v>
       </c>
       <c r="B50" t="s">
         <v>48</v>
       </c>
       <c r="C50" t="s">
-        <v>329</v>
+        <v>311</v>
       </c>
       <c r="D50" t="s">
         <v>152</v>
@@ -4507,18 +4542,18 @@
         <v>3</v>
       </c>
       <c r="F50" t="s">
-        <v>323</v>
+        <v>305</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
-        <v>324</v>
+        <v>306</v>
       </c>
       <c r="B51" t="s">
         <v>48</v>
       </c>
       <c r="C51" t="s">
-        <v>325</v>
+        <v>307</v>
       </c>
       <c r="D51" t="s">
         <v>152</v>
@@ -4527,18 +4562,18 @@
         <v>1</v>
       </c>
       <c r="F51" t="s">
-        <v>323</v>
+        <v>305</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
-        <v>332</v>
+        <v>314</v>
       </c>
       <c r="B52" t="s">
         <v>48</v>
       </c>
       <c r="C52" t="s">
-        <v>333</v>
+        <v>315</v>
       </c>
       <c r="D52" t="s">
         <v>152</v>
@@ -4547,18 +4582,18 @@
         <v>5</v>
       </c>
       <c r="F52" t="s">
-        <v>323</v>
+        <v>305</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
-        <v>316</v>
+        <v>298</v>
       </c>
       <c r="B53" t="s">
         <v>81</v>
       </c>
       <c r="C53" t="s">
-        <v>317</v>
+        <v>299</v>
       </c>
       <c r="D53" t="s">
         <v>152</v>
@@ -4567,18 +4602,18 @@
         <v>2</v>
       </c>
       <c r="F53" t="s">
-        <v>313</v>
+        <v>295</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
-        <v>318</v>
+        <v>300</v>
       </c>
       <c r="B54" t="s">
         <v>81</v>
       </c>
       <c r="C54" t="s">
-        <v>319</v>
+        <v>301</v>
       </c>
       <c r="D54" t="s">
         <v>152</v>
@@ -4587,18 +4622,18 @@
         <v>3</v>
       </c>
       <c r="F54" t="s">
-        <v>313</v>
+        <v>295</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
-        <v>314</v>
+        <v>296</v>
       </c>
       <c r="B55" t="s">
         <v>81</v>
       </c>
       <c r="C55" t="s">
-        <v>315</v>
+        <v>297</v>
       </c>
       <c r="D55" t="s">
         <v>152</v>
@@ -4607,18 +4642,18 @@
         <v>1</v>
       </c>
       <c r="F55" t="s">
-        <v>313</v>
+        <v>295</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
-        <v>320</v>
+        <v>302</v>
       </c>
       <c r="B56" t="s">
         <v>81</v>
       </c>
       <c r="C56" t="s">
-        <v>321</v>
+        <v>303</v>
       </c>
       <c r="D56" t="s">
         <v>152</v>
@@ -4627,12 +4662,12 @@
         <v>4</v>
       </c>
       <c r="F56" t="s">
-        <v>313</v>
+        <v>295</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
-        <v>312</v>
+        <v>294</v>
       </c>
       <c r="B57" t="s">
         <v>81</v>
@@ -4647,7 +4682,7 @@
         <v>0</v>
       </c>
       <c r="F57" t="s">
-        <v>313</v>
+        <v>295</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.45">
@@ -4678,7 +4713,7 @@
         <v>129</v>
       </c>
       <c r="C59" t="s">
-        <v>538</v>
+        <v>520</v>
       </c>
       <c r="D59" t="s">
         <v>152</v>
@@ -4718,7 +4753,7 @@
         <v>129</v>
       </c>
       <c r="C61" t="s">
-        <v>539</v>
+        <v>521</v>
       </c>
       <c r="D61" t="s">
         <v>152</v>
@@ -4738,7 +4773,7 @@
         <v>129</v>
       </c>
       <c r="C62" t="s">
-        <v>540</v>
+        <v>522</v>
       </c>
       <c r="D62" t="s">
         <v>152</v>
@@ -4778,7 +4813,7 @@
         <v>129</v>
       </c>
       <c r="C64" t="s">
-        <v>541</v>
+        <v>523</v>
       </c>
       <c r="D64" t="s">
         <v>152</v>
@@ -4792,7 +4827,7 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
-        <v>346</v>
+        <v>328</v>
       </c>
       <c r="B65" t="s">
         <v>91</v>
@@ -4807,18 +4842,18 @@
         <v>0</v>
       </c>
       <c r="F65" t="s">
-        <v>347</v>
+        <v>329</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
-        <v>350</v>
+        <v>332</v>
       </c>
       <c r="B66" t="s">
         <v>91</v>
       </c>
       <c r="C66" t="s">
-        <v>351</v>
+        <v>333</v>
       </c>
       <c r="D66" t="s">
         <v>152</v>
@@ -4827,18 +4862,18 @@
         <v>2</v>
       </c>
       <c r="F66" t="s">
-        <v>347</v>
+        <v>329</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
-        <v>354</v>
+        <v>336</v>
       </c>
       <c r="B67" t="s">
         <v>91</v>
       </c>
       <c r="C67" t="s">
-        <v>355</v>
+        <v>337</v>
       </c>
       <c r="D67" t="s">
         <v>152</v>
@@ -4847,18 +4882,18 @@
         <v>4</v>
       </c>
       <c r="F67" t="s">
-        <v>347</v>
+        <v>329</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
-        <v>356</v>
+        <v>338</v>
       </c>
       <c r="B68" t="s">
         <v>91</v>
       </c>
       <c r="C68" t="s">
-        <v>357</v>
+        <v>339</v>
       </c>
       <c r="D68" t="s">
         <v>152</v>
@@ -4867,18 +4902,18 @@
         <v>5</v>
       </c>
       <c r="F68" t="s">
-        <v>347</v>
+        <v>329</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
-        <v>352</v>
+        <v>334</v>
       </c>
       <c r="B69" t="s">
         <v>91</v>
       </c>
       <c r="C69" t="s">
-        <v>353</v>
+        <v>335</v>
       </c>
       <c r="D69" t="s">
         <v>152</v>
@@ -4887,18 +4922,18 @@
         <v>3</v>
       </c>
       <c r="F69" t="s">
-        <v>347</v>
+        <v>329</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
-        <v>348</v>
+        <v>330</v>
       </c>
       <c r="B70" t="s">
         <v>91</v>
       </c>
       <c r="C70" t="s">
-        <v>349</v>
+        <v>331</v>
       </c>
       <c r="D70" t="s">
         <v>152</v>
@@ -4907,21 +4942,21 @@
         <v>1</v>
       </c>
       <c r="F70" t="s">
-        <v>347</v>
+        <v>329</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="B71" t="s">
         <v>69</v>
       </c>
       <c r="C71" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="D71" t="s">
-        <v>152</v>
+        <v>10</v>
       </c>
       <c r="E71">
         <v>7</v>
@@ -4932,13 +4967,13 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B72" t="s">
         <v>69</v>
       </c>
       <c r="C72" t="s">
-        <v>168</v>
+        <v>524</v>
       </c>
       <c r="D72" t="s">
         <v>152</v>
@@ -4952,13 +4987,13 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B73" t="s">
         <v>69</v>
       </c>
       <c r="C73" t="s">
-        <v>170</v>
+        <v>525</v>
       </c>
       <c r="D73" t="s">
         <v>152</v>
@@ -4972,13 +5007,13 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B74" t="s">
         <v>69</v>
       </c>
       <c r="C74" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D74" t="s">
         <v>152</v>
@@ -4992,13 +5027,13 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B75" t="s">
         <v>69</v>
       </c>
       <c r="C75" t="s">
-        <v>174</v>
+        <v>526</v>
       </c>
       <c r="D75" t="s">
         <v>152</v>
@@ -5012,13 +5047,13 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B76" t="s">
         <v>69</v>
       </c>
       <c r="C76" t="s">
-        <v>166</v>
+        <v>527</v>
       </c>
       <c r="D76" t="s">
         <v>152</v>
@@ -5038,7 +5073,7 @@
         <v>69</v>
       </c>
       <c r="C77" t="s">
-        <v>164</v>
+        <v>528</v>
       </c>
       <c r="D77" t="s">
         <v>152</v>
@@ -5058,10 +5093,10 @@
         <v>69</v>
       </c>
       <c r="C78" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="D78" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E78">
         <v>0</v>
@@ -5072,13 +5107,13 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="B79" t="s">
         <v>76</v>
       </c>
       <c r="C79" t="s">
-        <v>202</v>
+        <v>532</v>
       </c>
       <c r="D79" t="s">
         <v>152</v>
@@ -5087,18 +5122,18 @@
         <v>3</v>
       </c>
       <c r="F79" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="B80" t="s">
         <v>76</v>
       </c>
       <c r="C80" t="s">
-        <v>206</v>
+        <v>190</v>
       </c>
       <c r="D80" t="s">
         <v>10</v>
@@ -5107,18 +5142,18 @@
         <v>5</v>
       </c>
       <c r="F80" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="B81" t="s">
         <v>76</v>
       </c>
       <c r="C81" t="s">
-        <v>200</v>
+        <v>533</v>
       </c>
       <c r="D81" t="s">
         <v>152</v>
@@ -5127,18 +5162,18 @@
         <v>2</v>
       </c>
       <c r="F81" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="B82" t="s">
         <v>76</v>
       </c>
       <c r="C82" t="s">
-        <v>208</v>
+        <v>534</v>
       </c>
       <c r="D82" t="s">
         <v>152</v>
@@ -5147,12 +5182,12 @@
         <v>6</v>
       </c>
       <c r="F82" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="B83" t="s">
         <v>76</v>
@@ -5167,18 +5202,18 @@
         <v>0</v>
       </c>
       <c r="F83" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="B84" t="s">
         <v>76</v>
       </c>
       <c r="C84" t="s">
-        <v>204</v>
+        <v>535</v>
       </c>
       <c r="D84" t="s">
         <v>152</v>
@@ -5187,18 +5222,18 @@
         <v>4</v>
       </c>
       <c r="F84" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="B85" t="s">
         <v>76</v>
       </c>
       <c r="C85" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="D85" t="s">
         <v>152</v>
@@ -5207,18 +5242,18 @@
         <v>1</v>
       </c>
       <c r="F85" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
-        <v>360</v>
+        <v>342</v>
       </c>
       <c r="B86" t="s">
         <v>56</v>
       </c>
       <c r="C86" t="s">
-        <v>361</v>
+        <v>343</v>
       </c>
       <c r="D86" t="s">
         <v>152</v>
@@ -5227,18 +5262,18 @@
         <v>1</v>
       </c>
       <c r="F86" t="s">
-        <v>359</v>
+        <v>341</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
-        <v>370</v>
+        <v>352</v>
       </c>
       <c r="B87" t="s">
         <v>56</v>
       </c>
       <c r="C87" t="s">
-        <v>371</v>
+        <v>353</v>
       </c>
       <c r="D87" t="s">
         <v>152</v>
@@ -5247,18 +5282,18 @@
         <v>6</v>
       </c>
       <c r="F87" t="s">
-        <v>359</v>
+        <v>341</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
-        <v>362</v>
+        <v>344</v>
       </c>
       <c r="B88" t="s">
         <v>56</v>
       </c>
       <c r="C88" t="s">
-        <v>363</v>
+        <v>345</v>
       </c>
       <c r="D88" t="s">
         <v>152</v>
@@ -5267,18 +5302,18 @@
         <v>2</v>
       </c>
       <c r="F88" t="s">
-        <v>359</v>
+        <v>341</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
-        <v>368</v>
+        <v>350</v>
       </c>
       <c r="B89" t="s">
         <v>56</v>
       </c>
       <c r="C89" t="s">
-        <v>369</v>
+        <v>351</v>
       </c>
       <c r="D89" t="s">
         <v>152</v>
@@ -5287,12 +5322,12 @@
         <v>5</v>
       </c>
       <c r="F89" t="s">
-        <v>359</v>
+        <v>341</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
-        <v>358</v>
+        <v>340</v>
       </c>
       <c r="B90" t="s">
         <v>56</v>
@@ -5307,18 +5342,18 @@
         <v>0</v>
       </c>
       <c r="F90" t="s">
-        <v>359</v>
+        <v>341</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
-        <v>374</v>
+        <v>356</v>
       </c>
       <c r="B91" t="s">
         <v>56</v>
       </c>
       <c r="C91" t="s">
-        <v>375</v>
+        <v>357</v>
       </c>
       <c r="D91" t="s">
         <v>152</v>
@@ -5327,18 +5362,18 @@
         <v>8</v>
       </c>
       <c r="F91" t="s">
-        <v>359</v>
+        <v>341</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
-        <v>364</v>
+        <v>346</v>
       </c>
       <c r="B92" t="s">
         <v>56</v>
       </c>
       <c r="C92" t="s">
-        <v>365</v>
+        <v>347</v>
       </c>
       <c r="D92" t="s">
         <v>152</v>
@@ -5347,18 +5382,18 @@
         <v>3</v>
       </c>
       <c r="F92" t="s">
-        <v>359</v>
+        <v>341</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
-        <v>378</v>
+        <v>360</v>
       </c>
       <c r="B93" t="s">
         <v>56</v>
       </c>
       <c r="C93" t="s">
-        <v>379</v>
+        <v>361</v>
       </c>
       <c r="D93" t="s">
         <v>152</v>
@@ -5367,18 +5402,18 @@
         <v>10</v>
       </c>
       <c r="F93" t="s">
-        <v>359</v>
+        <v>341</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A94" t="s">
-        <v>366</v>
+        <v>348</v>
       </c>
       <c r="B94" t="s">
         <v>56</v>
       </c>
       <c r="C94" t="s">
-        <v>367</v>
+        <v>349</v>
       </c>
       <c r="D94" t="s">
         <v>152</v>
@@ -5387,18 +5422,18 @@
         <v>4</v>
       </c>
       <c r="F94" t="s">
-        <v>359</v>
+        <v>341</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A95" t="s">
-        <v>372</v>
+        <v>354</v>
       </c>
       <c r="B95" t="s">
         <v>56</v>
       </c>
       <c r="C95" t="s">
-        <v>373</v>
+        <v>355</v>
       </c>
       <c r="D95" t="s">
         <v>152</v>
@@ -5407,18 +5442,18 @@
         <v>7</v>
       </c>
       <c r="F95" t="s">
-        <v>359</v>
+        <v>341</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
-        <v>376</v>
+        <v>358</v>
       </c>
       <c r="B96" t="s">
         <v>56</v>
       </c>
       <c r="C96" t="s">
-        <v>377</v>
+        <v>359</v>
       </c>
       <c r="D96" t="s">
         <v>152</v>
@@ -5427,18 +5462,18 @@
         <v>9</v>
       </c>
       <c r="F96" t="s">
-        <v>359</v>
+        <v>341</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
-        <v>428</v>
+        <v>410</v>
       </c>
       <c r="B97" t="s">
         <v>117</v>
       </c>
       <c r="C97" t="s">
-        <v>429</v>
+        <v>411</v>
       </c>
       <c r="D97" t="s">
         <v>152</v>
@@ -5447,18 +5482,18 @@
         <v>5</v>
       </c>
       <c r="F97" t="s">
-        <v>419</v>
+        <v>401</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
-        <v>422</v>
+        <v>404</v>
       </c>
       <c r="B98" t="s">
         <v>117</v>
       </c>
       <c r="C98" t="s">
-        <v>423</v>
+        <v>405</v>
       </c>
       <c r="D98" t="s">
         <v>152</v>
@@ -5467,18 +5502,18 @@
         <v>2</v>
       </c>
       <c r="F98" t="s">
-        <v>419</v>
+        <v>401</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A99" t="s">
-        <v>424</v>
+        <v>406</v>
       </c>
       <c r="B99" t="s">
         <v>117</v>
       </c>
       <c r="C99" t="s">
-        <v>425</v>
+        <v>407</v>
       </c>
       <c r="D99" t="s">
         <v>152</v>
@@ -5487,18 +5522,18 @@
         <v>3</v>
       </c>
       <c r="F99" t="s">
-        <v>419</v>
+        <v>401</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A100" t="s">
-        <v>426</v>
+        <v>408</v>
       </c>
       <c r="B100" t="s">
         <v>117</v>
       </c>
       <c r="C100" t="s">
-        <v>427</v>
+        <v>409</v>
       </c>
       <c r="D100" t="s">
         <v>152</v>
@@ -5507,12 +5542,12 @@
         <v>4</v>
       </c>
       <c r="F100" t="s">
-        <v>419</v>
+        <v>401</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A101" t="s">
-        <v>418</v>
+        <v>400</v>
       </c>
       <c r="B101" t="s">
         <v>117</v>
@@ -5527,18 +5562,18 @@
         <v>0</v>
       </c>
       <c r="F101" t="s">
-        <v>419</v>
+        <v>401</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A102" t="s">
-        <v>430</v>
+        <v>412</v>
       </c>
       <c r="B102" t="s">
         <v>117</v>
       </c>
       <c r="C102" t="s">
-        <v>431</v>
+        <v>413</v>
       </c>
       <c r="D102" t="s">
         <v>152</v>
@@ -5547,18 +5582,18 @@
         <v>6</v>
       </c>
       <c r="F102" t="s">
-        <v>419</v>
+        <v>401</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A103" t="s">
-        <v>420</v>
+        <v>402</v>
       </c>
       <c r="B103" t="s">
         <v>117</v>
       </c>
       <c r="C103" t="s">
-        <v>421</v>
+        <v>403</v>
       </c>
       <c r="D103" t="s">
         <v>152</v>
@@ -5567,258 +5602,258 @@
         <v>1</v>
       </c>
       <c r="F103" t="s">
-        <v>419</v>
+        <v>401</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A104" t="s">
-        <v>249</v>
+        <v>221</v>
       </c>
       <c r="B104" t="s">
         <v>27</v>
       </c>
       <c r="C104" t="s">
-        <v>250</v>
+        <v>33</v>
       </c>
       <c r="D104" t="s">
-        <v>152</v>
+        <v>10</v>
       </c>
       <c r="E104">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F104" t="s">
-        <v>240</v>
+        <v>222</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A105" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="B105" t="s">
         <v>27</v>
       </c>
       <c r="C105" t="s">
-        <v>244</v>
+        <v>224</v>
       </c>
       <c r="D105" t="s">
         <v>152</v>
       </c>
       <c r="E105">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F105" t="s">
-        <v>240</v>
+        <v>222</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A106" t="s">
-        <v>245</v>
+        <v>225</v>
       </c>
       <c r="B106" t="s">
         <v>27</v>
       </c>
       <c r="C106" t="s">
-        <v>246</v>
+        <v>226</v>
       </c>
       <c r="D106" t="s">
         <v>152</v>
       </c>
       <c r="E106">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F106" t="s">
-        <v>240</v>
+        <v>222</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A107" t="s">
-        <v>251</v>
+        <v>227</v>
       </c>
       <c r="B107" t="s">
         <v>27</v>
       </c>
       <c r="C107" t="s">
-        <v>252</v>
+        <v>228</v>
       </c>
       <c r="D107" t="s">
         <v>152</v>
       </c>
       <c r="E107">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F107" t="s">
-        <v>240</v>
+        <v>222</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A108" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="B108" t="s">
         <v>27</v>
       </c>
       <c r="C108" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="D108" t="s">
         <v>152</v>
       </c>
       <c r="E108">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F108" t="s">
-        <v>240</v>
+        <v>222</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A109" t="s">
-        <v>247</v>
+        <v>231</v>
       </c>
       <c r="B109" t="s">
         <v>27</v>
       </c>
       <c r="C109" t="s">
-        <v>248</v>
+        <v>232</v>
       </c>
       <c r="D109" t="s">
         <v>152</v>
       </c>
       <c r="E109">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F109" t="s">
-        <v>240</v>
+        <v>222</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A110" t="s">
-        <v>253</v>
+        <v>233</v>
       </c>
       <c r="B110" t="s">
         <v>27</v>
       </c>
       <c r="C110" t="s">
-        <v>254</v>
+        <v>234</v>
       </c>
       <c r="D110" t="s">
         <v>152</v>
       </c>
       <c r="E110">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F110" t="s">
-        <v>240</v>
+        <v>222</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A111" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="B111" t="s">
         <v>27</v>
       </c>
       <c r="C111" t="s">
-        <v>33</v>
+        <v>236</v>
       </c>
       <c r="D111" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E111">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F111" t="s">
-        <v>240</v>
+        <v>222</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A112" t="s">
-        <v>213</v>
+        <v>197</v>
       </c>
       <c r="B112" t="s">
         <v>107</v>
       </c>
       <c r="C112" t="s">
-        <v>214</v>
+        <v>111</v>
       </c>
       <c r="D112" t="s">
-        <v>152</v>
+        <v>10</v>
       </c>
       <c r="E112">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F112" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A113" t="s">
-        <v>223</v>
+        <v>199</v>
       </c>
       <c r="B113" t="s">
         <v>107</v>
       </c>
       <c r="C113" t="s">
-        <v>224</v>
+        <v>536</v>
       </c>
       <c r="D113" t="s">
         <v>152</v>
       </c>
       <c r="E113">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F113" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A114" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="B114" t="s">
         <v>107</v>
       </c>
       <c r="C114" t="s">
-        <v>111</v>
+        <v>537</v>
       </c>
       <c r="D114" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E114">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F114" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A115" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="B115" t="s">
         <v>107</v>
       </c>
       <c r="C115" t="s">
-        <v>212</v>
+        <v>538</v>
       </c>
       <c r="D115" t="s">
         <v>152</v>
       </c>
       <c r="E115">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F115" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A116" t="s">
-        <v>217</v>
+        <v>202</v>
       </c>
       <c r="B116" t="s">
         <v>107</v>
       </c>
       <c r="C116" t="s">
-        <v>218</v>
+        <v>539</v>
       </c>
       <c r="D116" t="s">
         <v>152</v>
@@ -5827,18 +5862,18 @@
         <v>4</v>
       </c>
       <c r="F116" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A117" t="s">
-        <v>219</v>
+        <v>203</v>
       </c>
       <c r="B117" t="s">
         <v>107</v>
       </c>
       <c r="C117" t="s">
-        <v>220</v>
+        <v>204</v>
       </c>
       <c r="D117" t="s">
         <v>152</v>
@@ -5847,18 +5882,18 @@
         <v>5</v>
       </c>
       <c r="F117" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A118" t="s">
-        <v>221</v>
+        <v>205</v>
       </c>
       <c r="B118" t="s">
         <v>107</v>
       </c>
       <c r="C118" t="s">
-        <v>222</v>
+        <v>206</v>
       </c>
       <c r="D118" t="s">
         <v>152</v>
@@ -5867,198 +5902,198 @@
         <v>6</v>
       </c>
       <c r="F118" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A119" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="B119" t="s">
         <v>107</v>
       </c>
       <c r="C119" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="D119" t="s">
         <v>152</v>
       </c>
       <c r="E119">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F119" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A120" t="s">
-        <v>282</v>
+        <v>252</v>
       </c>
       <c r="B120" t="s">
         <v>43</v>
       </c>
       <c r="C120" t="s">
-        <v>283</v>
+        <v>47</v>
       </c>
       <c r="D120" t="s">
-        <v>152</v>
+        <v>10</v>
       </c>
       <c r="E120">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F120" t="s">
-        <v>271</v>
+        <v>253</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A121" t="s">
-        <v>278</v>
+        <v>254</v>
       </c>
       <c r="B121" t="s">
         <v>43</v>
       </c>
       <c r="C121" t="s">
-        <v>279</v>
+        <v>255</v>
       </c>
       <c r="D121" t="s">
         <v>152</v>
       </c>
       <c r="E121">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F121" t="s">
-        <v>271</v>
+        <v>253</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A122" t="s">
-        <v>276</v>
+        <v>256</v>
       </c>
       <c r="B122" t="s">
         <v>43</v>
       </c>
       <c r="C122" t="s">
-        <v>277</v>
+        <v>257</v>
       </c>
       <c r="D122" t="s">
         <v>152</v>
       </c>
       <c r="E122">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F122" t="s">
-        <v>271</v>
+        <v>253</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A123" t="s">
-        <v>280</v>
+        <v>258</v>
       </c>
       <c r="B123" t="s">
         <v>43</v>
       </c>
       <c r="C123" t="s">
-        <v>281</v>
+        <v>259</v>
       </c>
       <c r="D123" t="s">
         <v>152</v>
       </c>
       <c r="E123">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F123" t="s">
-        <v>271</v>
+        <v>253</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A124" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="B124" t="s">
         <v>43</v>
       </c>
       <c r="C124" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
       <c r="D124" t="s">
         <v>152</v>
       </c>
       <c r="E124">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F124" t="s">
-        <v>271</v>
+        <v>253</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A125" t="s">
-        <v>284</v>
+        <v>262</v>
       </c>
       <c r="B125" t="s">
         <v>43</v>
       </c>
       <c r="C125" t="s">
-        <v>285</v>
+        <v>263</v>
       </c>
       <c r="D125" t="s">
         <v>152</v>
       </c>
       <c r="E125">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F125" t="s">
-        <v>271</v>
+        <v>253</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A126" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="B126" t="s">
         <v>43</v>
       </c>
       <c r="C126" t="s">
-        <v>275</v>
+        <v>265</v>
       </c>
       <c r="D126" t="s">
         <v>152</v>
       </c>
       <c r="E126">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F126" t="s">
-        <v>271</v>
+        <v>253</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A127" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="B127" t="s">
         <v>43</v>
       </c>
       <c r="C127" t="s">
-        <v>47</v>
+        <v>267</v>
       </c>
       <c r="D127" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E127">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F127" t="s">
-        <v>271</v>
+        <v>253</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A128" t="s">
-        <v>446</v>
+        <v>428</v>
       </c>
       <c r="B128" t="s">
         <v>134</v>
       </c>
       <c r="C128" t="s">
-        <v>447</v>
+        <v>429</v>
       </c>
       <c r="D128" t="s">
         <v>152</v>
@@ -6067,18 +6102,18 @@
         <v>7</v>
       </c>
       <c r="F128" t="s">
-        <v>433</v>
+        <v>415</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A129" t="s">
-        <v>444</v>
+        <v>426</v>
       </c>
       <c r="B129" t="s">
         <v>134</v>
       </c>
       <c r="C129" t="s">
-        <v>445</v>
+        <v>427</v>
       </c>
       <c r="D129" t="s">
         <v>152</v>
@@ -6087,18 +6122,18 @@
         <v>6</v>
       </c>
       <c r="F129" t="s">
-        <v>433</v>
+        <v>415</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A130" t="s">
-        <v>434</v>
+        <v>416</v>
       </c>
       <c r="B130" t="s">
         <v>134</v>
       </c>
       <c r="C130" t="s">
-        <v>435</v>
+        <v>417</v>
       </c>
       <c r="D130" t="s">
         <v>152</v>
@@ -6107,12 +6142,12 @@
         <v>1</v>
       </c>
       <c r="F130" t="s">
-        <v>433</v>
+        <v>415</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A131" t="s">
-        <v>432</v>
+        <v>414</v>
       </c>
       <c r="B131" t="s">
         <v>134</v>
@@ -6127,18 +6162,18 @@
         <v>0</v>
       </c>
       <c r="F131" t="s">
-        <v>433</v>
+        <v>415</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A132" t="s">
-        <v>438</v>
+        <v>420</v>
       </c>
       <c r="B132" t="s">
         <v>134</v>
       </c>
       <c r="C132" t="s">
-        <v>439</v>
+        <v>421</v>
       </c>
       <c r="D132" t="s">
         <v>152</v>
@@ -6147,18 +6182,18 @@
         <v>3</v>
       </c>
       <c r="F132" t="s">
-        <v>433</v>
+        <v>415</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A133" t="s">
-        <v>442</v>
+        <v>424</v>
       </c>
       <c r="B133" t="s">
         <v>134</v>
       </c>
       <c r="C133" t="s">
-        <v>443</v>
+        <v>425</v>
       </c>
       <c r="D133" t="s">
         <v>152</v>
@@ -6167,18 +6202,18 @@
         <v>5</v>
       </c>
       <c r="F133" t="s">
-        <v>433</v>
+        <v>415</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A134" t="s">
-        <v>436</v>
+        <v>418</v>
       </c>
       <c r="B134" t="s">
         <v>134</v>
       </c>
       <c r="C134" t="s">
-        <v>437</v>
+        <v>419</v>
       </c>
       <c r="D134" t="s">
         <v>152</v>
@@ -6187,18 +6222,18 @@
         <v>2</v>
       </c>
       <c r="F134" t="s">
-        <v>433</v>
+        <v>415</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A135" t="s">
-        <v>440</v>
+        <v>422</v>
       </c>
       <c r="B135" t="s">
         <v>134</v>
       </c>
       <c r="C135" t="s">
-        <v>441</v>
+        <v>423</v>
       </c>
       <c r="D135" t="s">
         <v>152</v>
@@ -6207,353 +6242,353 @@
         <v>4</v>
       </c>
       <c r="F135" t="s">
-        <v>433</v>
+        <v>415</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A136" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="B136" t="s">
         <v>141</v>
       </c>
       <c r="C136" t="s">
-        <v>188</v>
+        <v>529</v>
       </c>
       <c r="D136" t="s">
-        <v>152</v>
+        <v>10</v>
       </c>
       <c r="E136">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F136" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A137" t="s">
-        <v>191</v>
+        <v>174</v>
       </c>
       <c r="B137" t="s">
         <v>141</v>
       </c>
       <c r="C137" t="s">
-        <v>192</v>
+        <v>530</v>
       </c>
       <c r="D137" t="s">
         <v>152</v>
       </c>
       <c r="E137">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F137" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A138" t="s">
-        <v>193</v>
+        <v>175</v>
       </c>
       <c r="B138" t="s">
         <v>141</v>
       </c>
       <c r="C138" t="s">
-        <v>194</v>
+        <v>531</v>
       </c>
       <c r="D138" t="s">
         <v>152</v>
       </c>
       <c r="E138">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F138" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A139" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B139" t="s">
         <v>141</v>
       </c>
       <c r="C139" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="D139" t="s">
         <v>152</v>
       </c>
       <c r="E139">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F139" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A140" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B140" t="s">
         <v>141</v>
       </c>
       <c r="C140" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D140" t="s">
         <v>152</v>
       </c>
       <c r="E140">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F140" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A141" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B141" t="s">
         <v>141</v>
       </c>
       <c r="C141" t="s">
-        <v>145</v>
+        <v>182</v>
       </c>
       <c r="D141" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E141">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F141" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A142" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B142" t="s">
         <v>141</v>
       </c>
       <c r="C142" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D142" t="s">
         <v>152</v>
       </c>
       <c r="E142">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F142" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A143" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B143" t="s">
         <v>141</v>
       </c>
       <c r="C143" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D143" t="s">
         <v>152</v>
       </c>
       <c r="E143">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F143" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A144" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B144" t="s">
         <v>141</v>
       </c>
       <c r="C144" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D144" t="s">
         <v>152</v>
       </c>
       <c r="E144">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F144" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A145" t="s">
-        <v>266</v>
+        <v>237</v>
       </c>
       <c r="B145" t="s">
         <v>35</v>
       </c>
       <c r="C145" t="s">
-        <v>267</v>
+        <v>41</v>
       </c>
       <c r="D145" t="s">
-        <v>152</v>
+        <v>10</v>
       </c>
       <c r="E145">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F145" t="s">
-        <v>256</v>
+        <v>238</v>
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A146" t="s">
-        <v>261</v>
+        <v>239</v>
       </c>
       <c r="B146" t="s">
         <v>35</v>
       </c>
       <c r="C146" t="s">
-        <v>262</v>
+        <v>240</v>
       </c>
       <c r="D146" t="s">
         <v>152</v>
       </c>
       <c r="E146">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F146" t="s">
-        <v>256</v>
+        <v>238</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A147" t="s">
-        <v>257</v>
+        <v>241</v>
       </c>
       <c r="B147" t="s">
         <v>35</v>
       </c>
       <c r="C147" t="s">
-        <v>258</v>
+        <v>242</v>
       </c>
       <c r="D147" t="s">
         <v>152</v>
       </c>
       <c r="E147">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F147" t="s">
-        <v>256</v>
+        <v>238</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A148" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="B148" t="s">
         <v>35</v>
       </c>
       <c r="C148" t="s">
-        <v>264</v>
+        <v>244</v>
       </c>
       <c r="D148" t="s">
         <v>152</v>
       </c>
       <c r="E148">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F148" t="s">
-        <v>256</v>
+        <v>238</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A149" t="s">
-        <v>268</v>
+        <v>245</v>
       </c>
       <c r="B149" t="s">
         <v>35</v>
       </c>
       <c r="C149" t="s">
-        <v>269</v>
+        <v>246</v>
       </c>
       <c r="D149" t="s">
         <v>152</v>
       </c>
       <c r="E149">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F149" t="s">
-        <v>256</v>
+        <v>238</v>
       </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A150" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="B150" t="s">
         <v>35</v>
       </c>
       <c r="C150" t="s">
-        <v>41</v>
+        <v>246</v>
       </c>
       <c r="D150" t="s">
-        <v>10</v>
+        <v>152</v>
       </c>
       <c r="E150">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F150" t="s">
-        <v>256</v>
+        <v>238</v>
       </c>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A151" t="s">
-        <v>265</v>
+        <v>248</v>
       </c>
       <c r="B151" t="s">
         <v>35</v>
       </c>
       <c r="C151" t="s">
-        <v>264</v>
+        <v>249</v>
       </c>
       <c r="D151" t="s">
         <v>152</v>
       </c>
       <c r="E151">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F151" t="s">
-        <v>256</v>
+        <v>238</v>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A152" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="B152" t="s">
         <v>35</v>
       </c>
       <c r="C152" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="D152" t="s">
         <v>152</v>
       </c>
       <c r="E152">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F152" t="s">
-        <v>256</v>
+        <v>238</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1" xr:uid="{00000000-0009-0000-0000-000002000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F152">
-      <sortCondition ref="B1"/>
+  <autoFilter ref="A1:F152" xr:uid="{00000000-0009-0000-0000-000002000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A8:F14">
+      <sortCondition ref="E1:E152"/>
     </sortState>
   </autoFilter>
   <hyperlinks>
@@ -6561,9 +6596,24 @@
     <hyperlink ref="C60" r:id="rId2" xr:uid="{2C3D556D-39AA-4885-AD25-D636D5148266}"/>
     <hyperlink ref="C61" r:id="rId3" xr:uid="{8AA99DC7-365F-46C5-809B-E7D4E69A9EDF}"/>
     <hyperlink ref="C63" r:id="rId4" xr:uid="{368E5479-408D-4DE9-814B-B19BEA995149}"/>
+    <hyperlink ref="C71" r:id="rId5" xr:uid="{DF281175-B0DD-4262-9A1B-6E40746866ED}"/>
+    <hyperlink ref="C74" r:id="rId6" xr:uid="{7A1BA145-5FB5-4A16-AB53-1192C8FEC1ED}"/>
+    <hyperlink ref="C78" r:id="rId7" xr:uid="{AA0D7652-1F49-46F2-83CB-3BEAE1ABFD22}"/>
+    <hyperlink ref="C139" r:id="rId8" xr:uid="{99098D5E-4E17-4CFF-AE1A-C04D902CBCEA}"/>
+    <hyperlink ref="C140" r:id="rId9" xr:uid="{32757D02-7D6D-4D50-9031-C9135006C939}"/>
+    <hyperlink ref="C141" r:id="rId10" xr:uid="{B35054F2-14B8-47DA-A285-E51E57BBB218}"/>
+    <hyperlink ref="C142" r:id="rId11" xr:uid="{6FB74026-B363-4A94-9AC2-8B5AFB388E95}"/>
+    <hyperlink ref="C143" r:id="rId12" xr:uid="{B80E1A9B-48C8-4FC1-819E-069E59701FF4}"/>
+    <hyperlink ref="C144" r:id="rId13" xr:uid="{1160C1A0-BCB1-44CF-A33F-2B54CD035F48}"/>
+    <hyperlink ref="C80" r:id="rId14" xr:uid="{39AC63DE-91A7-4BA8-9748-6AF075816BA2}"/>
+    <hyperlink ref="C85" r:id="rId15" xr:uid="{3EF882F6-0CFD-4863-BA94-B07FBD3230F7}"/>
+    <hyperlink ref="C112" r:id="rId16" xr:uid="{A1B00CD2-6799-4655-987B-FEB4D7AC3415}"/>
+    <hyperlink ref="C109" r:id="rId17" xr:uid="{9F7F9644-58B2-4E5D-8673-8FFF24E28052}"/>
+    <hyperlink ref="C104" r:id="rId18" xr:uid="{0571A7FE-348C-4782-9D60-DBC8398BE283}"/>
+    <hyperlink ref="C151" r:id="rId19" xr:uid="{E7806D70-E3CE-4197-8A28-280D41F372C8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId20"/>
 </worksheet>
 </file>
 
@@ -6594,58 +6644,58 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>448</v>
+        <v>430</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>449</v>
+        <v>431</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>450</v>
+        <v>432</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>451</v>
+        <v>433</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>452</v>
+        <v>434</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>453</v>
+        <v>435</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>454</v>
+        <v>436</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>455</v>
+        <v>437</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>456</v>
+        <v>438</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>457</v>
+        <v>439</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>458</v>
+        <v>440</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>459</v>
+        <v>441</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>460</v>
+        <v>442</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>461</v>
+        <v>443</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>462</v>
+        <v>444</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>463</v>
+        <v>445</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>464</v>
+        <v>446</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>465</v>
+        <v>447</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>6</v>
@@ -6656,61 +6706,61 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>506</v>
+        <v>488</v>
       </c>
       <c r="B2" t="s">
-        <v>507</v>
+        <v>489</v>
       </c>
       <c r="C2" t="s">
-        <v>508</v>
+        <v>490</v>
       </c>
       <c r="D2" t="s">
-        <v>509</v>
+        <v>491</v>
       </c>
       <c r="E2" t="s">
-        <v>510</v>
+        <v>492</v>
       </c>
       <c r="F2" t="s">
-        <v>511</v>
+        <v>493</v>
       </c>
       <c r="G2" t="s">
-        <v>512</v>
+        <v>494</v>
       </c>
       <c r="H2" t="s">
-        <v>513</v>
+        <v>495</v>
       </c>
       <c r="I2" t="s">
-        <v>514</v>
+        <v>496</v>
       </c>
       <c r="J2" t="s">
-        <v>515</v>
+        <v>497</v>
       </c>
       <c r="K2" t="s">
-        <v>516</v>
+        <v>498</v>
       </c>
       <c r="L2" t="s">
-        <v>517</v>
+        <v>499</v>
       </c>
       <c r="M2" t="s">
-        <v>518</v>
+        <v>500</v>
       </c>
       <c r="N2" t="s">
         <v>138</v>
       </c>
       <c r="O2" t="s">
-        <v>519</v>
+        <v>501</v>
       </c>
       <c r="P2" t="s">
         <v>139</v>
       </c>
       <c r="Q2" t="s">
-        <v>520</v>
+        <v>502</v>
       </c>
       <c r="T2" t="s">
-        <v>521</v>
+        <v>503</v>
       </c>
       <c r="U2" t="s">
-        <v>522</v>
+        <v>504</v>
       </c>
     </row>
   </sheetData>
@@ -6739,22 +6789,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>466</v>
+        <v>448</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>448</v>
+        <v>430</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>146</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>467</v>
+        <v>449</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>468</v>
+        <v>450</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>469</v>
+        <v>451</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>6</v>
@@ -6762,13 +6812,13 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>523</v>
+        <v>505</v>
       </c>
       <c r="B2" t="s">
+        <v>488</v>
+      </c>
+      <c r="C2" t="s">
         <v>506</v>
-      </c>
-      <c r="C2" t="s">
-        <v>524</v>
       </c>
       <c r="D2" t="s">
         <v>136</v>
@@ -6780,7 +6830,7 @@
         <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>521</v>
+        <v>503</v>
       </c>
     </row>
   </sheetData>
@@ -6807,16 +6857,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>466</v>
+        <v>448</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>448</v>
+        <v>430</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>458</v>
+        <v>440</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>470</v>
+        <v>452</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>6</v>
@@ -6824,70 +6874,70 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>525</v>
+        <v>507</v>
       </c>
       <c r="B2" t="s">
-        <v>506</v>
+        <v>488</v>
       </c>
       <c r="C2" t="s">
-        <v>526</v>
+        <v>508</v>
       </c>
       <c r="D2" t="s">
-        <v>527</v>
+        <v>509</v>
       </c>
       <c r="E2" t="s">
-        <v>521</v>
+        <v>503</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>528</v>
+        <v>510</v>
       </c>
       <c r="B3" t="s">
-        <v>506</v>
+        <v>488</v>
       </c>
       <c r="C3" t="s">
-        <v>529</v>
+        <v>511</v>
       </c>
       <c r="D3" t="s">
-        <v>530</v>
+        <v>512</v>
       </c>
       <c r="E3" t="s">
-        <v>531</v>
+        <v>513</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>532</v>
+        <v>514</v>
       </c>
       <c r="B4" t="s">
-        <v>506</v>
+        <v>488</v>
       </c>
       <c r="C4" t="s">
-        <v>533</v>
+        <v>515</v>
       </c>
       <c r="D4" t="s">
-        <v>534</v>
+        <v>516</v>
       </c>
       <c r="E4" t="s">
-        <v>535</v>
+        <v>517</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>536</v>
+        <v>518</v>
       </c>
       <c r="B5" t="s">
-        <v>506</v>
+        <v>488</v>
       </c>
       <c r="C5" t="s">
-        <v>517</v>
+        <v>499</v>
       </c>
       <c r="D5" t="s">
-        <v>537</v>
+        <v>519</v>
       </c>
       <c r="E5" t="s">
-        <v>522</v>
+        <v>504</v>
       </c>
     </row>
   </sheetData>
@@ -6915,19 +6965,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>471</v>
+        <v>453</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>472</v>
+        <v>454</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>473</v>
+        <v>455</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>474</v>
+        <v>456</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>6</v>
@@ -6938,22 +6988,22 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>475</v>
+        <v>457</v>
       </c>
       <c r="B2" t="s">
-        <v>476</v>
+        <v>458</v>
       </c>
       <c r="C2" t="s">
-        <v>477</v>
+        <v>459</v>
       </c>
       <c r="D2" t="s">
-        <v>478</v>
+        <v>460</v>
       </c>
       <c r="E2" t="s">
         <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>479</v>
+        <v>461</v>
       </c>
       <c r="G2" t="s">
         <v>11</v>
@@ -6981,18 +7031,18 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>480</v>
+        <v>462</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>481</v>
+        <v>463</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>482</v>
+        <v>464</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -7003,7 +7053,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>482</v>
+        <v>464</v>
       </c>
       <c r="B3">
         <v>4</v>
@@ -7014,7 +7064,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>482</v>
+        <v>464</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -7025,7 +7075,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>482</v>
+        <v>464</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -7036,233 +7086,233 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B6" t="s">
         <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>484</v>
+        <v>466</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B7" t="s">
         <v>35</v>
       </c>
       <c r="C7" t="s">
-        <v>485</v>
+        <v>467</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B8" t="s">
         <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>486</v>
+        <v>468</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B9" t="s">
         <v>48</v>
       </c>
       <c r="C9" t="s">
-        <v>487</v>
+        <v>469</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B10" t="s">
         <v>56</v>
       </c>
       <c r="C10" t="s">
-        <v>488</v>
+        <v>470</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B11" t="s">
         <v>62</v>
       </c>
       <c r="C11" t="s">
-        <v>489</v>
+        <v>471</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B12" t="s">
         <v>69</v>
       </c>
       <c r="C12" t="s">
-        <v>490</v>
+        <v>472</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B13" t="s">
         <v>76</v>
       </c>
       <c r="C13" t="s">
-        <v>491</v>
+        <v>473</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B14" t="s">
         <v>81</v>
       </c>
       <c r="C14" t="s">
-        <v>492</v>
+        <v>474</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B15" t="s">
         <v>85</v>
       </c>
       <c r="C15" t="s">
-        <v>493</v>
+        <v>475</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B16" t="s">
         <v>91</v>
       </c>
       <c r="C16" t="s">
-        <v>494</v>
+        <v>476</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B17" t="s">
         <v>96</v>
       </c>
       <c r="C17" t="s">
-        <v>495</v>
+        <v>477</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B18" t="s">
         <v>101</v>
       </c>
       <c r="C18" t="s">
-        <v>496</v>
+        <v>478</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B19" t="s">
         <v>107</v>
       </c>
       <c r="C19" t="s">
-        <v>497</v>
+        <v>479</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B20" t="s">
         <v>112</v>
       </c>
       <c r="C20" t="s">
-        <v>498</v>
+        <v>480</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B21" t="s">
         <v>117</v>
       </c>
       <c r="C21" t="s">
-        <v>499</v>
+        <v>481</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B22" t="s">
         <v>124</v>
       </c>
       <c r="C22" t="s">
-        <v>500</v>
+        <v>482</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B23" t="s">
         <v>129</v>
       </c>
       <c r="C23" t="s">
-        <v>501</v>
+        <v>483</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B24" t="s">
         <v>134</v>
       </c>
       <c r="C24" t="s">
-        <v>502</v>
+        <v>484</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>483</v>
+        <v>465</v>
       </c>
       <c r="B25" t="s">
         <v>141</v>
       </c>
       <c r="C25" t="s">
-        <v>503</v>
+        <v>485</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>504</v>
+        <v>486</v>
       </c>
       <c r="B26" t="s">
-        <v>475</v>
+        <v>457</v>
       </c>
       <c r="C26" t="s">
-        <v>505</v>
+        <v>487</v>
       </c>
     </row>
   </sheetData>

</xml_diff>